<commit_message>
reordered files, plots updated
</commit_message>
<xml_diff>
--- a/scripts/Model_Stats.xlsx
+++ b/scripts/Model_Stats.xlsx
@@ -1,18 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29225"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29227"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8EC7DDB2-AEF8-4982-A612-DAB798136A3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6899C17C-AD00-4CC8-8E3B-C96402D2A9CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Img_Class" sheetId="1" r:id="rId1"/>
     <sheet name="Obj_Det" sheetId="2" r:id="rId2"/>
     <sheet name="Segmentation" sheetId="3" r:id="rId3"/>
-    <sheet name="Audio_Classification" sheetId="4" r:id="rId4"/>
-    <sheet name="Sheet1" sheetId="5" r:id="rId5"/>
+    <sheet name="Segmentation (2)" sheetId="6" r:id="rId4"/>
+    <sheet name="Audio_Classification" sheetId="4" r:id="rId5"/>
+    <sheet name="Sheet1" sheetId="5" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="90">
   <si>
     <t>Model name</t>
   </si>
@@ -128,6 +129,12 @@
     <t>MobileNet V3</t>
   </si>
   <si>
+    <t>Model Name</t>
+  </si>
+  <si>
+    <t>mAP</t>
+  </si>
+  <si>
     <t>SSD MobileNet V1</t>
   </si>
   <si>
@@ -135,9 +142,6 @@
 COCO</t>
   </si>
   <si>
-    <t>6.5 ms</t>
-  </si>
-  <si>
     <t>Yes</t>
   </si>
   <si>
@@ -147,18 +151,12 @@
     <t>SSD MobileNet V2(TF1)</t>
   </si>
   <si>
-    <t>7.3 ms</t>
-  </si>
-  <si>
     <t>6.6 MB</t>
   </si>
   <si>
     <t>SSD MobileNet V2 (TF2)</t>
   </si>
   <si>
-    <t>7.6 ms</t>
-  </si>
-  <si>
     <t>6.7 MB</t>
   </si>
   <si>
@@ -171,13 +169,7 @@
     <t>320x320x3</t>
   </si>
   <si>
-    <t>5.2 ms</t>
-  </si>
-  <si>
     <t>SSDLite MobileDet</t>
-  </si>
-  <si>
-    <t>9.1 ms</t>
   </si>
   <si>
     <t>5.1 MB</t>
@@ -444,7 +436,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -480,36 +472,12 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF888888"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF888888"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF888888"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF888888"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF888888"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -527,13 +495,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -917,7 +878,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="36">
+    <row r="2" spans="1:9" ht="29.25">
       <c r="A2" s="1" t="s">
         <v>9</v>
       </c>
@@ -946,7 +907,7 @@
         <v>12.8</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="36">
+    <row r="3" spans="1:9" ht="29.25">
       <c r="A3" s="1" t="s">
         <v>13</v>
       </c>
@@ -975,7 +936,7 @@
         <v>8.6999999999999993</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="36">
+    <row r="4" spans="1:9" ht="29.25">
       <c r="A4" s="1" t="s">
         <v>15</v>
       </c>
@@ -1316,253 +1277,148 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDB0845C-31B8-42AA-BA89-221D7425A0A4}">
-  <dimension ref="A3:G20"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20.28515625" customWidth="1"/>
     <col min="2" max="2" width="16.5703125" customWidth="1"/>
     <col min="3" max="3" width="17" customWidth="1"/>
+    <col min="4" max="4" width="13.28515625" customWidth="1"/>
     <col min="5" max="5" width="12.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:7" ht="29.25">
+    <row r="1" spans="1:7">
+      <c r="A1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="29.25">
+      <c r="A2" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="3">
+        <v>6.5</v>
+      </c>
+      <c r="E2" s="3">
+        <v>21.5</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="36">
       <c r="A3" s="1" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D3" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="E3" s="9">
-        <v>21.5</v>
+      <c r="D3" s="3">
+        <v>7.3</v>
+      </c>
+      <c r="E3" s="3">
+        <v>25.6</v>
       </c>
       <c r="F3" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="36">
+      <c r="A4" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="C4" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" s="3">
+        <v>7.6</v>
+      </c>
+      <c r="E4" s="3">
+        <v>22.4</v>
+      </c>
+      <c r="F4" s="3" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="4" spans="1:7">
-      <c r="A4" s="7"/>
-      <c r="B4" s="7"/>
-      <c r="C4" s="7"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="10"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7"/>
-    </row>
-    <row r="5" spans="1:7">
-      <c r="A5" s="7"/>
-      <c r="B5" s="7"/>
-      <c r="C5" s="7"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="10"/>
-      <c r="F5" s="7"/>
-      <c r="G5" s="7"/>
-    </row>
-    <row r="6" spans="1:7">
-      <c r="A6" s="8"/>
-      <c r="B6" s="8"/>
-      <c r="C6" s="8"/>
-      <c r="D6" s="8"/>
-      <c r="E6" s="11"/>
-      <c r="F6" s="8"/>
-      <c r="G6" s="8"/>
-    </row>
-    <row r="7" spans="1:7" ht="36">
-      <c r="A7" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="E7" s="9">
-        <v>25.6</v>
-      </c>
-      <c r="F7" s="3" t="s">
+      <c r="G4" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="17.25">
+      <c r="A5" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D5" s="3">
+        <v>5.2</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="29.25">
+      <c r="A6" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="G7" s="3" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7">
-      <c r="A8" s="7"/>
-      <c r="B8" s="7"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="10"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="7"/>
-    </row>
-    <row r="9" spans="1:7">
-      <c r="A9" s="7"/>
-      <c r="B9" s="7"/>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="10"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="7"/>
-    </row>
-    <row r="10" spans="1:7">
-      <c r="A10" s="8"/>
-      <c r="B10" s="8"/>
-      <c r="C10" s="8"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="11"/>
-      <c r="F10" s="8"/>
-      <c r="G10" s="8"/>
-    </row>
-    <row r="11" spans="1:7" ht="36">
-      <c r="A11" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="E11" s="9">
-        <v>22.4</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="G11" s="3" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7">
-      <c r="A12" s="7"/>
-      <c r="B12" s="7"/>
-      <c r="C12" s="7"/>
-      <c r="D12" s="7"/>
-      <c r="E12" s="10"/>
-      <c r="F12" s="7"/>
-      <c r="G12" s="7"/>
-    </row>
-    <row r="13" spans="1:7">
-      <c r="A13" s="8"/>
-      <c r="B13" s="8"/>
-      <c r="C13" s="8"/>
-      <c r="D13" s="8"/>
-      <c r="E13" s="11"/>
-      <c r="F13" s="8"/>
-      <c r="G13" s="8"/>
-    </row>
-    <row r="14" spans="1:7" ht="17.25">
-      <c r="A14" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="B14" s="1" t="s">
+      <c r="C6" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="C14" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="D14" s="3" t="s">
+      <c r="D6" s="3">
+        <v>9.1</v>
+      </c>
+      <c r="E6" s="3">
+        <v>32.9</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G6" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="E14" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="F14" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="G14" s="3" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7">
-      <c r="A15" s="7"/>
-      <c r="B15" s="7"/>
-      <c r="C15" s="7"/>
-      <c r="D15" s="7"/>
-      <c r="E15" s="10"/>
-      <c r="F15" s="7"/>
-      <c r="G15" s="7"/>
-    </row>
-    <row r="16" spans="1:7">
-      <c r="A16" s="8"/>
-      <c r="B16" s="8"/>
-      <c r="C16" s="8"/>
-      <c r="D16" s="8"/>
-      <c r="E16" s="11"/>
-      <c r="F16" s="8"/>
-      <c r="G16" s="8"/>
-    </row>
-    <row r="17" spans="1:7" ht="29.25">
-      <c r="A17" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="D17" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="E17" s="9">
-        <v>32.9</v>
-      </c>
-      <c r="F17" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="G17" s="3" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7">
-      <c r="A18" s="7"/>
-      <c r="B18" s="7"/>
-      <c r="C18" s="7"/>
-      <c r="D18" s="7"/>
-      <c r="E18" s="10"/>
-      <c r="F18" s="7"/>
-      <c r="G18" s="7"/>
-    </row>
-    <row r="19" spans="1:7">
-      <c r="A19" s="7"/>
-      <c r="B19" s="7"/>
-      <c r="C19" s="7"/>
-      <c r="D19" s="7"/>
-      <c r="E19" s="10"/>
-      <c r="F19" s="7"/>
-      <c r="G19" s="7"/>
-    </row>
-    <row r="20" spans="1:7">
-      <c r="A20" s="8"/>
-      <c r="B20" s="8"/>
-      <c r="C20" s="8"/>
-      <c r="D20" s="8"/>
-      <c r="E20" s="8"/>
-      <c r="F20" s="8"/>
-      <c r="G20" s="8"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B3" r:id="rId1" xr:uid="{46F32AAE-FB10-4510-9EEF-BC43822B8FFF}"/>
-    <hyperlink ref="B7" r:id="rId2" xr:uid="{FE4C6CC1-6766-4F55-85BA-9896C9CD36DC}"/>
-    <hyperlink ref="B11" r:id="rId3" xr:uid="{D7D39AF2-AF76-41F4-90DA-B7288346BFA7}"/>
-    <hyperlink ref="B17" r:id="rId4" xr:uid="{8ED3DD2F-6D64-4DED-826F-040CA8FC7CA4}"/>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{46F32AAE-FB10-4510-9EEF-BC43822B8FFF}"/>
+    <hyperlink ref="B3" r:id="rId2" xr:uid="{FE4C6CC1-6766-4F55-85BA-9896C9CD36DC}"/>
+    <hyperlink ref="B4" r:id="rId3" xr:uid="{D7D39AF2-AF76-41F4-90DA-B7288346BFA7}"/>
+    <hyperlink ref="B6" r:id="rId4" xr:uid="{8ED3DD2F-6D64-4DED-826F-040CA8FC7CA4}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1570,7 +1426,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B423EC3-4326-4D86-A2CF-3A05129F67CD}">
-  <dimension ref="A1:J14"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="29.28515625" customWidth="1"/>
@@ -1581,25 +1437,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
+      <c r="A1" t="s">
+        <v>30</v>
+      </c>
       <c r="C1" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D1" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="H1" t="s">
         <v>5</v>
       </c>
       <c r="J1" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="29.25">
       <c r="A2" s="1" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>20</v>
@@ -1618,21 +1477,21 @@
         <v>2.7</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="29.25">
       <c r="A3" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>51</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>54</v>
       </c>
       <c r="D3" s="3"/>
       <c r="E3" s="3" t="s">
@@ -1648,268 +1507,40 @@
         <v>29</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="J3" s="3" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="17.25">
+      <c r="A4" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="C4" s="8" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="4" spans="1:10" ht="17.25">
-      <c r="A4" s="12" t="s">
+      <c r="D4" s="8"/>
+      <c r="E4" s="8">
+        <v>0.75</v>
+      </c>
+      <c r="F4" s="8">
+        <v>16</v>
+      </c>
+      <c r="G4" s="8">
+        <v>1</v>
+      </c>
+      <c r="H4" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="I4" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="J4" s="8" t="s">
         <v>56</v>
-      </c>
-      <c r="B4" s="12" t="s">
-        <v>57</v>
-      </c>
-      <c r="C4" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="D4" s="13"/>
-      <c r="E4" s="13">
-        <v>0.75</v>
-      </c>
-      <c r="F4" s="13">
-        <v>16</v>
-      </c>
-      <c r="G4" s="13">
-        <v>1</v>
-      </c>
-      <c r="H4" s="13" t="s">
-        <v>12</v>
-      </c>
-      <c r="I4" s="13" t="s">
-        <v>33</v>
-      </c>
-      <c r="J4" s="13" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" ht="17.25">
-      <c r="A5" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3">
-        <v>0.75</v>
-      </c>
-      <c r="F5" s="3">
-        <v>16</v>
-      </c>
-      <c r="G5" s="3">
-        <v>1</v>
-      </c>
-      <c r="H5" s="3">
-        <v>6.9</v>
-      </c>
-      <c r="I5" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="J5" s="3" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10">
-      <c r="A6" s="8"/>
-      <c r="B6" s="8"/>
-      <c r="C6" s="8"/>
-      <c r="D6" s="8"/>
-      <c r="E6" s="8"/>
-      <c r="F6" s="8"/>
-      <c r="G6" s="8"/>
-      <c r="H6" s="8"/>
-      <c r="I6" s="8"/>
-      <c r="J6" s="8"/>
-    </row>
-    <row r="7" spans="1:10" ht="17.25">
-      <c r="A7" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3">
-        <v>0.75</v>
-      </c>
-      <c r="F7" s="3">
-        <v>16</v>
-      </c>
-      <c r="G7" s="3">
-        <v>1</v>
-      </c>
-      <c r="H7" s="3">
-        <v>10.7</v>
-      </c>
-      <c r="I7" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="J7" s="3" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10">
-      <c r="A8" s="8"/>
-      <c r="B8" s="8"/>
-      <c r="C8" s="8"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="8"/>
-      <c r="F8" s="8"/>
-      <c r="G8" s="8"/>
-      <c r="H8" s="8"/>
-      <c r="I8" s="8"/>
-      <c r="J8" s="8"/>
-    </row>
-    <row r="9" spans="1:10" ht="17.25">
-      <c r="A9" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3">
-        <v>0.75</v>
-      </c>
-      <c r="F9" s="3">
-        <v>16</v>
-      </c>
-      <c r="G9" s="3">
-        <v>1</v>
-      </c>
-      <c r="H9" s="3">
-        <v>12.3</v>
-      </c>
-      <c r="I9" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="J9" s="3" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10">
-      <c r="A10" s="8"/>
-      <c r="B10" s="8"/>
-      <c r="C10" s="8"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="8"/>
-      <c r="F10" s="8"/>
-      <c r="G10" s="8"/>
-      <c r="H10" s="8"/>
-      <c r="I10" s="8"/>
-      <c r="J10" s="8"/>
-    </row>
-    <row r="11" spans="1:10" ht="17.25">
-      <c r="A11" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3">
-        <v>0.75</v>
-      </c>
-      <c r="F11" s="3">
-        <v>16</v>
-      </c>
-      <c r="G11" s="3">
-        <v>1</v>
-      </c>
-      <c r="H11" s="3">
-        <v>17.7</v>
-      </c>
-      <c r="I11" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="J11" s="3" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10">
-      <c r="A12" s="8"/>
-      <c r="B12" s="8"/>
-      <c r="C12" s="8"/>
-      <c r="D12" s="8"/>
-      <c r="E12" s="8"/>
-      <c r="F12" s="8"/>
-      <c r="G12" s="8"/>
-      <c r="H12" s="8"/>
-      <c r="I12" s="8"/>
-      <c r="J12" s="8"/>
-    </row>
-    <row r="13" spans="1:10" ht="17.25">
-      <c r="A13" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="D13" s="3"/>
-      <c r="E13" s="3">
-        <v>0.75</v>
-      </c>
-      <c r="F13" s="3">
-        <v>16</v>
-      </c>
-      <c r="G13" s="3">
-        <v>1</v>
-      </c>
-      <c r="H13" s="3">
-        <v>30.8</v>
-      </c>
-      <c r="I13" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="J13" s="3" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" ht="17.25">
-      <c r="A14" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3">
-        <v>0.75</v>
-      </c>
-      <c r="F14" s="3">
-        <v>16</v>
-      </c>
-      <c r="G14" s="3">
-        <v>1</v>
-      </c>
-      <c r="H14" s="3">
-        <v>38.799999999999997</v>
-      </c>
-      <c r="I14" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="J14" s="3" t="s">
-        <v>70</v>
       </c>
     </row>
   </sheetData>
@@ -1922,6 +1553,314 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA0E4EB4-541C-40BA-A77A-994BF8F1E900}">
+  <dimension ref="A1:J10"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="29.28515625" customWidth="1"/>
+    <col min="2" max="2" width="21.42578125" customWidth="1"/>
+    <col min="3" max="4" width="16.85546875" customWidth="1"/>
+    <col min="8" max="8" width="14.7109375" customWidth="1"/>
+    <col min="10" max="10" width="12" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10">
+      <c r="A1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D1" t="s">
+        <v>46</v>
+      </c>
+      <c r="H1" t="s">
+        <v>5</v>
+      </c>
+      <c r="J1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="29.25">
+      <c r="A2" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G2" s="3">
+        <v>1</v>
+      </c>
+      <c r="H2" s="3">
+        <v>2.7</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="29.25">
+      <c r="A3" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G3" s="3">
+        <v>1</v>
+      </c>
+      <c r="H3" s="3">
+        <v>29</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="17.25">
+      <c r="A4" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="D4" s="8"/>
+      <c r="E4" s="8">
+        <v>0.75</v>
+      </c>
+      <c r="F4" s="8">
+        <v>16</v>
+      </c>
+      <c r="G4" s="8">
+        <v>1</v>
+      </c>
+      <c r="H4" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="I4" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="J4" s="8" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="17.25">
+      <c r="A5" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3">
+        <v>0.75</v>
+      </c>
+      <c r="F5" s="3">
+        <v>16</v>
+      </c>
+      <c r="G5" s="3">
+        <v>1</v>
+      </c>
+      <c r="H5" s="3">
+        <v>6.9</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="17.25">
+      <c r="A6" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3">
+        <v>0.75</v>
+      </c>
+      <c r="F6" s="3">
+        <v>16</v>
+      </c>
+      <c r="G6" s="3">
+        <v>1</v>
+      </c>
+      <c r="H6" s="3">
+        <v>10.7</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="J6" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="17.25">
+      <c r="A7" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3">
+        <v>0.75</v>
+      </c>
+      <c r="F7" s="3">
+        <v>16</v>
+      </c>
+      <c r="G7" s="3">
+        <v>1</v>
+      </c>
+      <c r="H7" s="3">
+        <v>12.3</v>
+      </c>
+      <c r="I7" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="J7" s="3" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="17.25">
+      <c r="A8" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3">
+        <v>0.75</v>
+      </c>
+      <c r="F8" s="3">
+        <v>16</v>
+      </c>
+      <c r="G8" s="3">
+        <v>1</v>
+      </c>
+      <c r="H8" s="3">
+        <v>17.7</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="J8" s="3" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="17.25">
+      <c r="A9" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3">
+        <v>0.75</v>
+      </c>
+      <c r="F9" s="3">
+        <v>16</v>
+      </c>
+      <c r="G9" s="3">
+        <v>1</v>
+      </c>
+      <c r="H9" s="3">
+        <v>30.8</v>
+      </c>
+      <c r="I9" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="J9" s="3" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="17.25">
+      <c r="A10" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3">
+        <v>0.75</v>
+      </c>
+      <c r="F10" s="3">
+        <v>16</v>
+      </c>
+      <c r="G10" s="3">
+        <v>1</v>
+      </c>
+      <c r="H10" s="3">
+        <v>38.799999999999997</v>
+      </c>
+      <c r="I10" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="J10" s="3" t="s">
+        <v>67</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{FDF0FBDC-362F-44A4-95A9-ACCF3795F05B}"/>
+    <hyperlink ref="B3" r:id="rId2" xr:uid="{661BC6EE-6720-44F4-8113-ED7EE7D88FF3}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D27D2D4-349F-4FDE-A36B-C526DD467D49}">
   <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1942,73 +1881,73 @@
         <v>2</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="E1" s="4" t="s">
         <v>8</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="70.5">
       <c r="A2" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="E2" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="F2" s="6" t="s">
         <v>74</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="F2" s="6" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="70.5">
       <c r="A3" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="E3" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>81</v>
-      </c>
       <c r="F3" s="6" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="70.5">
       <c r="A4" s="1" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
   </sheetData>
@@ -2021,7 +1960,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14BFF91C-8706-47A5-8CF3-9E5386477F76}">
   <dimension ref="A1:H5"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2046,56 +1985,56 @@
         <v>2</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="H1" s="4" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="36">
-      <c r="A2" s="12" t="s">
-        <v>86</v>
-      </c>
-      <c r="B2" s="12" t="s">
-        <v>87</v>
-      </c>
-      <c r="C2" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="D2" s="13">
+      <c r="A2" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="D2" s="8">
         <v>16</v>
       </c>
-      <c r="E2" s="13">
-        <v>1</v>
-      </c>
-      <c r="F2" s="13" t="s">
+      <c r="E2" s="8">
+        <v>1</v>
+      </c>
+      <c r="F2" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="13" t="s">
-        <v>33</v>
-      </c>
-      <c r="H2" s="13" t="s">
-        <v>59</v>
+      <c r="G2" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="H2" s="8" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="36">
       <c r="A3" s="1" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="D3" s="3">
         <v>16</v>
@@ -2107,21 +2046,21 @@
         <v>5.8</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="36">
       <c r="A4" s="1" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C4" s="3" t="s">
         <v>87</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>90</v>
       </c>
       <c r="D4" s="3">
         <v>16</v>
@@ -2133,21 +2072,21 @@
         <v>10.3</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="36">
       <c r="A5" s="1" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D5" s="3">
         <v>16</v>
@@ -2159,10 +2098,10 @@
         <v>32.4</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fixed plotting bugs, single model testing
</commit_message>
<xml_diff>
--- a/scripts/Model_Stats.xlsx
+++ b/scripts/Model_Stats.xlsx
@@ -26,10 +26,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="13">
+  <fonts count="11">
     <font>
       <name val="Aptos Narrow"/>
-      <charset val="1"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
@@ -51,30 +50,26 @@
     </font>
     <font>
       <name val="Inherit"/>
-      <charset val="1"/>
       <family val="0"/>
       <b val="1"/>
-      <color rgb="FF4A4A4A"/>
+      <color theme="1"/>
       <sz val="12"/>
     </font>
     <font>
       <name val="inherit"/>
-      <charset val="1"/>
       <family val="0"/>
       <b val="1"/>
-      <color rgb="FF4A4A4A"/>
+      <color theme="1"/>
       <sz val="12"/>
     </font>
     <font>
       <name val="Brown Light"/>
-      <charset val="1"/>
       <family val="0"/>
-      <color rgb="FF4A4A4A"/>
+      <color theme="1"/>
       <sz val="12"/>
     </font>
     <font>
       <name val="Aptos Narrow"/>
-      <charset val="1"/>
       <family val="2"/>
       <color theme="10"/>
       <sz val="11"/>
@@ -82,28 +77,15 @@
     </font>
     <font>
       <name val="Inherit"/>
-      <charset val="1"/>
       <family val="0"/>
-      <color rgb="FF4A4A4A"/>
+      <color theme="1"/>
       <sz val="12"/>
     </font>
     <font>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
-    </font>
-    <font>
       <name val="Cambria"/>
-      <charset val="1"/>
       <family val="0"/>
       <b val="1"/>
+      <color theme="1"/>
       <sz val="11"/>
     </font>
     <font>
@@ -180,7 +162,7 @@
       <bottom style="thin"/>
     </border>
   </borders>
-  <cellStyleXfs count="7">
+  <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -189,11 +171,11 @@
     <xf numFmtId="44" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1">
+  </cellStyleXfs>
+  <cellXfs count="25">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
-  </cellStyleXfs>
-  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -203,13 +185,10 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="bottom"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="20">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -218,13 +197,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -233,7 +209,7 @@
     <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="20">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -249,19 +225,13 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="20">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -270,21 +240,20 @@
     <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="20">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
-  <cellStyles count="7">
+  <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Comma [0]" xfId="2" builtinId="6"/>
     <cellStyle name="Currency" xfId="3" builtinId="4"/>
     <cellStyle name="Currency [0]" xfId="4" builtinId="7"/>
     <cellStyle name="Percent" xfId="5" builtinId="5"/>
-    <cellStyle name="*unknown*" xfId="6" builtinId="8"/>
   </cellStyles>
   <dxfs count="13">
     <dxf>
@@ -498,14 +467,14 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="020F0302020204030204" pitchFamily="0" charset="1"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204" pitchFamily="0" charset="1"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme>
@@ -513,67 +482,25 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill>
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:tint val="67000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:tint val="73000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:tint val="81000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
-        </a:gradFill>
-        <a:gradFill>
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:shade val="78000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
-        </a:gradFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
+          <a:miter/>
         </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
+          <a:miter/>
         </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
+          <a:miter/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
@@ -592,35 +519,11 @@
           <a:schemeClr val="phClr"/>
         </a:solidFill>
         <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-          </a:schemeClr>
+          <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill>
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
-        </a:gradFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
@@ -636,654 +539,654 @@
   <dimension ref="A1:K14"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="29.86" customWidth="1" style="14" min="1" max="1"/>
-    <col width="22" customWidth="1" style="14" min="2" max="2"/>
-    <col width="17.57" customWidth="1" style="14" min="3" max="3"/>
-    <col width="12.14" customWidth="1" style="14" min="4" max="4"/>
-    <col width="11.86" customWidth="1" style="14" min="5" max="5"/>
-    <col width="15.72" customWidth="1" style="14" min="6" max="6"/>
-    <col width="15" customWidth="1" style="14" min="7" max="7"/>
-    <col width="21.01" customWidth="1" style="14" min="8" max="8"/>
-    <col width="21.59" customWidth="1" style="14" min="9" max="9"/>
-    <col width="25.86" customWidth="1" style="14" min="10" max="10"/>
-    <col width="31.22" customWidth="1" style="14" min="11" max="11"/>
+    <col width="29.86" customWidth="1" style="13" min="1" max="1"/>
+    <col width="24.39" customWidth="1" style="13" min="2" max="2"/>
+    <col width="17.57" customWidth="1" style="13" min="3" max="3"/>
+    <col width="12.14" customWidth="1" style="13" min="4" max="4"/>
+    <col width="11.86" customWidth="1" style="13" min="5" max="5"/>
+    <col width="15.72" customWidth="1" style="13" min="6" max="6"/>
+    <col width="15" customWidth="1" style="13" min="7" max="7"/>
+    <col width="21.01" customWidth="1" style="13" min="8" max="8"/>
+    <col width="21.59" customWidth="1" style="13" min="9" max="9"/>
+    <col width="25.86" customWidth="1" style="13" min="10" max="10"/>
+    <col width="31.22" customWidth="1" style="13" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row r="1" ht="36" customHeight="1" s="15">
-      <c r="A1" s="16" t="inlineStr">
+    <row r="1" ht="36" customHeight="1" s="14">
+      <c r="A1" s="15" t="inlineStr">
         <is>
           <t>Model name</t>
         </is>
       </c>
-      <c r="B1" s="16" t="inlineStr">
+      <c r="B1" s="15" t="inlineStr">
         <is>
           <t>Detections/Dataset</t>
         </is>
       </c>
-      <c r="C1" s="16" t="inlineStr">
+      <c r="C1" s="15" t="inlineStr">
         <is>
           <t>Input size</t>
         </is>
       </c>
-      <c r="D1" s="16" t="inlineStr">
+      <c r="D1" s="15" t="inlineStr">
         <is>
           <t>Depth mul.</t>
         </is>
       </c>
-      <c r="E1" s="16" t="inlineStr">
+      <c r="E1" s="15" t="inlineStr">
         <is>
           <t>TF ver.</t>
         </is>
       </c>
-      <c r="F1" s="17" t="inlineStr">
+      <c r="F1" s="16" t="inlineStr">
         <is>
           <t>Latency (ms)</t>
         </is>
       </c>
-      <c r="G1" s="16" t="inlineStr">
+      <c r="G1" s="15" t="inlineStr">
         <is>
           <t>Top-1 Accuracy</t>
         </is>
       </c>
-      <c r="H1" s="16" t="inlineStr">
+      <c r="H1" s="15" t="inlineStr">
         <is>
           <t>Top-5 Accuracy</t>
         </is>
       </c>
-      <c r="I1" s="16" t="inlineStr">
+      <c r="I1" s="15" t="inlineStr">
         <is>
           <t>Model size</t>
         </is>
       </c>
-      <c r="J1" s="14" t="inlineStr">
+      <c r="J1" s="13" t="inlineStr">
         <is>
           <t>Measured-Quoted (ms)</t>
         </is>
       </c>
-      <c r="K1" s="14" t="inlineStr">
+      <c r="K1" s="13" t="inlineStr">
         <is>
           <t>% Difference</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="29.25" customHeight="1" s="15">
-      <c r="A2" s="18" t="inlineStr">
+    <row r="2" ht="29.25" customHeight="1" s="14">
+      <c r="A2" s="17" t="inlineStr">
         <is>
           <t>EfficientNet-EdgeTpu (L)</t>
         </is>
       </c>
-      <c r="B2" s="19" t="inlineStr">
+      <c r="B2" s="18" t="inlineStr">
         <is>
           <t>1,000 objects
 ILSVRC2012</t>
         </is>
       </c>
-      <c r="C2" s="20" t="inlineStr">
+      <c r="C2" s="19" t="inlineStr">
         <is>
           <t>300x300x3</t>
         </is>
       </c>
-      <c r="D2" s="20" t="inlineStr">
+      <c r="D2" s="19" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="E2" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="F2" s="20" t="n">
+      <c r="E2" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" s="19" t="n">
         <v>21.3</v>
       </c>
-      <c r="G2" s="20" t="n">
+      <c r="G2" s="19" t="n">
         <v>81.2</v>
       </c>
-      <c r="H2" s="20" t="n">
+      <c r="H2" s="19" t="n">
         <v>95.09999999999999</v>
       </c>
-      <c r="I2" s="20" t="n">
+      <c r="I2" s="19" t="n">
         <v>12.8</v>
       </c>
-      <c r="J2" s="14">
+      <c r="J2" s="13">
         <f>Img_Class_outs!E13-F2</f>
         <v/>
       </c>
-      <c r="K2" s="14">
+      <c r="K2" s="13">
         <f>J2/F2 * 100</f>
         <v/>
       </c>
     </row>
-    <row r="3" ht="29.25" customHeight="1" s="15">
-      <c r="A3" s="18" t="inlineStr">
+    <row r="3" ht="29.25" customHeight="1" s="14">
+      <c r="A3" s="17" t="inlineStr">
         <is>
           <t>EfficientNet-EdgeTpu (M)</t>
         </is>
       </c>
-      <c r="B3" s="19" t="inlineStr">
+      <c r="B3" s="18" t="inlineStr">
         <is>
           <t>1,000 objects
 ILSVRC2012</t>
         </is>
       </c>
-      <c r="C3" s="20" t="inlineStr">
+      <c r="C3" s="19" t="inlineStr">
         <is>
           <t>240x240x3</t>
         </is>
       </c>
-      <c r="D3" s="20" t="inlineStr">
+      <c r="D3" s="19" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="E3" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="F3" s="20" t="n">
+      <c r="E3" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" s="19" t="n">
         <v>7.3</v>
       </c>
-      <c r="G3" s="20" t="n">
+      <c r="G3" s="19" t="n">
         <v>80.09999999999999</v>
       </c>
-      <c r="H3" s="20" t="n">
+      <c r="H3" s="19" t="n">
         <v>94.5</v>
       </c>
-      <c r="I3" s="20" t="n">
+      <c r="I3" s="19" t="n">
         <v>8.699999999999999</v>
       </c>
-      <c r="J3" s="14">
+      <c r="J3" s="13">
         <f>Img_Class_outs!E12-F3</f>
         <v/>
       </c>
-      <c r="K3" s="14">
+      <c r="K3" s="13">
         <f>J3/F3 * 100</f>
         <v/>
       </c>
     </row>
-    <row r="4" ht="29.25" customHeight="1" s="15">
-      <c r="A4" s="18" t="inlineStr">
+    <row r="4" ht="29.25" customHeight="1" s="14">
+      <c r="A4" s="17" t="inlineStr">
         <is>
           <t>EfficientNet-EdgeTpu (S)</t>
         </is>
       </c>
-      <c r="B4" s="19" t="inlineStr">
+      <c r="B4" s="18" t="inlineStr">
         <is>
           <t>1,000 objects
 ILSVRC2012</t>
         </is>
       </c>
-      <c r="C4" s="20" t="inlineStr">
+      <c r="C4" s="19" t="inlineStr">
         <is>
           <t>224x224x3</t>
         </is>
       </c>
-      <c r="D4" s="20" t="inlineStr">
+      <c r="D4" s="19" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="E4" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="F4" s="20" t="n">
+      <c r="E4" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" s="19" t="n">
         <v>5</v>
       </c>
-      <c r="G4" s="20" t="n">
+      <c r="G4" s="19" t="n">
         <v>78.90000000000001</v>
       </c>
-      <c r="H4" s="20" t="n">
+      <c r="H4" s="19" t="n">
         <v>94.7</v>
       </c>
-      <c r="I4" s="20" t="n">
+      <c r="I4" s="19" t="n">
         <v>6.8</v>
       </c>
-      <c r="J4" s="14">
+      <c r="J4" s="13">
         <f>Img_Class_outs!E10-F4</f>
         <v/>
       </c>
-      <c r="K4" s="14">
+      <c r="K4" s="13">
         <f>J4/F4 * 100</f>
         <v/>
       </c>
     </row>
-    <row r="5" ht="29.25" customHeight="1" s="15">
-      <c r="A5" s="18" t="inlineStr">
+    <row r="5" ht="29.25" customHeight="1" s="14">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>Inception V1</t>
         </is>
       </c>
-      <c r="B5" s="19" t="inlineStr">
+      <c r="B5" s="18" t="inlineStr">
         <is>
           <t>1,000 objects
 ILSVRC2012</t>
         </is>
       </c>
-      <c r="C5" s="20" t="inlineStr">
+      <c r="C5" s="19" t="inlineStr">
         <is>
           <t>224x224x3</t>
         </is>
       </c>
-      <c r="D5" s="20" t="inlineStr">
+      <c r="D5" s="19" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="E5" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="F5" s="20" t="n">
+      <c r="E5" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" s="19" t="n">
         <v>3.4</v>
       </c>
-      <c r="G5" s="20" t="n">
+      <c r="G5" s="19" t="n">
         <v>71.90000000000001</v>
       </c>
-      <c r="H5" s="20" t="n">
+      <c r="H5" s="19" t="n">
         <v>92</v>
       </c>
-      <c r="I5" s="20" t="n">
+      <c r="I5" s="19" t="n">
         <v>7</v>
       </c>
-      <c r="J5" s="21">
+      <c r="J5" s="13">
         <f>Img_Class_outs!E11 - F5</f>
         <v/>
       </c>
-      <c r="K5" s="14">
+      <c r="K5" s="13">
         <f>J5/F5 * 100</f>
         <v/>
       </c>
     </row>
-    <row r="6" ht="29.25" customHeight="1" s="15">
-      <c r="A6" s="18" t="inlineStr">
+    <row r="6" ht="29.25" customHeight="1" s="14">
+      <c r="A6" s="17" t="inlineStr">
         <is>
           <t>Inception V3</t>
         </is>
       </c>
-      <c r="B6" s="19" t="inlineStr">
+      <c r="B6" s="18" t="inlineStr">
         <is>
           <t>1,000 objects
 ILSVRC2012</t>
         </is>
       </c>
-      <c r="C6" s="20" t="inlineStr">
+      <c r="C6" s="19" t="inlineStr">
         <is>
           <t>224x224x3</t>
         </is>
       </c>
-      <c r="D6" s="20" t="inlineStr">
+      <c r="D6" s="19" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="E6" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="F6" s="20" t="n">
+      <c r="E6" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" s="19" t="n">
         <v>13.4</v>
       </c>
-      <c r="G6" s="20" t="n">
+      <c r="G6" s="19" t="n">
         <v>75.40000000000001</v>
       </c>
-      <c r="H6" s="20" t="n">
+      <c r="H6" s="19" t="n">
         <v>93.2</v>
       </c>
-      <c r="I6" s="20" t="n">
+      <c r="I6" s="19" t="n">
         <v>12</v>
       </c>
-      <c r="J6" s="14">
+      <c r="J6" s="13">
         <f>Img_Class_outs!E14 - F6</f>
         <v/>
       </c>
-      <c r="K6" s="14">
+      <c r="K6" s="13">
         <f>J6/F6 * 100</f>
         <v/>
       </c>
     </row>
-    <row r="7" ht="29.25" customHeight="1" s="15">
-      <c r="A7" s="18" t="inlineStr">
+    <row r="7" ht="29.25" customHeight="1" s="14">
+      <c r="A7" s="17" t="inlineStr">
         <is>
           <t>MobileNet V1 (0.25)</t>
         </is>
       </c>
-      <c r="B7" s="19" t="inlineStr">
+      <c r="B7" s="18" t="inlineStr">
         <is>
           <t>1,000 objects
 ILSVRC2012</t>
         </is>
       </c>
-      <c r="C7" s="20" t="inlineStr">
+      <c r="C7" s="19" t="inlineStr">
         <is>
           <t>128x128x3</t>
         </is>
       </c>
-      <c r="D7" s="20" t="n">
+      <c r="D7" s="19" t="n">
         <v>0.25</v>
       </c>
-      <c r="E7" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="F7" s="20" t="n">
+      <c r="E7" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" s="19" t="n">
         <v>0.9</v>
       </c>
-      <c r="G7" s="20" t="n">
+      <c r="G7" s="19" t="n">
         <v>40.8</v>
       </c>
-      <c r="H7" s="20" t="n">
+      <c r="H7" s="19" t="n">
         <v>67.2</v>
       </c>
-      <c r="I7" s="20" t="n">
+      <c r="I7" s="19" t="n">
         <v>0.7</v>
       </c>
-      <c r="J7" s="22">
+      <c r="J7" s="13">
         <f>Img_Class_outs!E2-F7</f>
         <v/>
       </c>
-      <c r="K7" s="14">
+      <c r="K7" s="13">
         <f>J7/F7 * 100</f>
         <v/>
       </c>
     </row>
-    <row r="8" ht="29.25" customHeight="1" s="15">
-      <c r="A8" s="18" t="inlineStr">
+    <row r="8" ht="29.25" customHeight="1" s="14">
+      <c r="A8" s="17" t="inlineStr">
         <is>
           <t>MobileNet V1 (0.50)</t>
         </is>
       </c>
-      <c r="B8" s="19" t="inlineStr">
+      <c r="B8" s="18" t="inlineStr">
         <is>
           <t>1,000 objects
 ILSVRC2012</t>
         </is>
       </c>
-      <c r="C8" s="20" t="inlineStr">
+      <c r="C8" s="19" t="inlineStr">
         <is>
           <t>160x160x3</t>
         </is>
       </c>
-      <c r="D8" s="20" t="n">
+      <c r="D8" s="19" t="n">
         <v>0.5</v>
       </c>
-      <c r="E8" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="F8" s="20" t="n">
+      <c r="E8" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" s="19" t="n">
         <v>1.4</v>
       </c>
-      <c r="G8" s="20" t="n">
+      <c r="G8" s="19" t="n">
         <v>63.7</v>
       </c>
-      <c r="H8" s="20" t="n">
+      <c r="H8" s="19" t="n">
         <v>83.40000000000001</v>
       </c>
-      <c r="I8" s="20" t="n">
+      <c r="I8" s="19" t="n">
         <v>1.6</v>
       </c>
-      <c r="J8" s="22">
+      <c r="J8" s="13">
         <f>Img_Class_outs!E3-F8</f>
         <v/>
       </c>
-      <c r="K8" s="14">
+      <c r="K8" s="13">
         <f>J8/F8 * 100</f>
         <v/>
       </c>
     </row>
-    <row r="9" ht="29.25" customHeight="1" s="15">
-      <c r="A9" s="18" t="inlineStr">
+    <row r="9" ht="29.25" customHeight="1" s="14">
+      <c r="A9" s="17" t="inlineStr">
         <is>
           <t>MobileNet V1 (.75)</t>
         </is>
       </c>
-      <c r="B9" s="19" t="inlineStr">
+      <c r="B9" s="18" t="inlineStr">
         <is>
           <t>1,000 objects
 ILSVRC2012</t>
         </is>
       </c>
-      <c r="C9" s="20" t="inlineStr">
+      <c r="C9" s="19" t="inlineStr">
         <is>
           <t>192x192x3</t>
         </is>
       </c>
-      <c r="D9" s="20" t="n">
+      <c r="D9" s="19" t="n">
         <v>0.75</v>
       </c>
-      <c r="E9" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="F9" s="20" t="n">
+      <c r="E9" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" s="19" t="n">
         <v>1.8</v>
       </c>
-      <c r="G9" s="20" t="n">
+      <c r="G9" s="19" t="n">
         <v>67.2</v>
       </c>
-      <c r="H9" s="20" t="n">
+      <c r="H9" s="19" t="n">
         <v>88.09999999999999</v>
       </c>
-      <c r="I9" s="20" t="n">
+      <c r="I9" s="19" t="n">
         <v>2.8</v>
       </c>
-      <c r="J9" s="22">
+      <c r="J9" s="13">
         <f>Img_Class_outs!E4-F9</f>
         <v/>
       </c>
-      <c r="K9" s="14">
+      <c r="K9" s="13">
         <f>J9/F9 * 100</f>
         <v/>
       </c>
     </row>
-    <row r="10" ht="29.25" customHeight="1" s="15">
-      <c r="A10" s="18" t="inlineStr">
+    <row r="10" ht="29.25" customHeight="1" s="14">
+      <c r="A10" s="17" t="inlineStr">
         <is>
           <t>MobileNet V1 (1.0)</t>
         </is>
       </c>
-      <c r="B10" s="19" t="inlineStr">
+      <c r="B10" s="18" t="inlineStr">
         <is>
           <t>1,000 objects
 ILSVRC2012</t>
         </is>
       </c>
-      <c r="C10" s="20" t="inlineStr">
+      <c r="C10" s="19" t="inlineStr">
         <is>
           <t>224x224x3</t>
         </is>
       </c>
-      <c r="D10" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="E10" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="F10" s="20" t="n">
+      <c r="D10" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" s="19" t="n">
         <v>2.8</v>
       </c>
-      <c r="G10" s="20" t="n">
+      <c r="G10" s="19" t="n">
         <v>69.5</v>
       </c>
-      <c r="H10" s="20" t="n">
+      <c r="H10" s="19" t="n">
         <v>90.59999999999999</v>
       </c>
-      <c r="I10" s="20" t="n">
+      <c r="I10" s="19" t="n">
         <v>4.4</v>
       </c>
-      <c r="J10" s="22">
+      <c r="J10" s="13">
         <f>Img_Class_outs!E5-F10</f>
         <v/>
       </c>
-      <c r="K10" s="14">
+      <c r="K10" s="13">
         <f>J10/F10 * 100</f>
         <v/>
       </c>
     </row>
-    <row r="11" ht="29.25" customHeight="1" s="15">
-      <c r="A11" s="18" t="inlineStr">
+    <row r="11" ht="29.25" customHeight="1" s="14">
+      <c r="A11" s="17" t="inlineStr">
         <is>
           <t>MobileNet V1 (TF_ver_2.0)</t>
         </is>
       </c>
-      <c r="B11" s="19" t="inlineStr">
+      <c r="B11" s="18" t="inlineStr">
         <is>
           <t>1,000 objects
 ILSVRC2012</t>
         </is>
       </c>
-      <c r="C11" s="20" t="inlineStr">
+      <c r="C11" s="19" t="inlineStr">
         <is>
           <t>224x224x3</t>
         </is>
       </c>
-      <c r="D11" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="E11" s="20" t="n">
+      <c r="D11" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="19" t="n">
         <v>2</v>
       </c>
-      <c r="F11" s="20" t="n">
+      <c r="F11" s="19" t="n">
         <v>2.8</v>
       </c>
-      <c r="G11" s="20" t="n">
+      <c r="G11" s="19" t="n">
         <v>69.5</v>
       </c>
-      <c r="H11" s="20" t="n">
+      <c r="H11" s="19" t="n">
         <v>89.8</v>
       </c>
-      <c r="I11" s="20" t="n">
+      <c r="I11" s="19" t="n">
         <v>4.5</v>
       </c>
-      <c r="J11" s="14">
+      <c r="J11" s="13">
         <f>Img_Class_outs!E9-F11</f>
         <v/>
       </c>
-      <c r="K11" s="14">
+      <c r="K11" s="13">
         <f>J11/F11 * 100</f>
         <v/>
       </c>
     </row>
-    <row r="12" ht="29.25" customHeight="1" s="15">
-      <c r="A12" s="18" t="inlineStr">
+    <row r="12" ht="29.25" customHeight="1" s="14">
+      <c r="A12" s="17" t="inlineStr">
         <is>
           <t>MobileNet V2</t>
         </is>
       </c>
-      <c r="B12" s="19" t="inlineStr">
+      <c r="B12" s="18" t="inlineStr">
         <is>
           <t>1,000 objects
 ILSVRC2012</t>
         </is>
       </c>
-      <c r="C12" s="20" t="inlineStr">
+      <c r="C12" s="19" t="inlineStr">
         <is>
           <t>224x224x3</t>
         </is>
       </c>
-      <c r="D12" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="E12" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="F12" s="20" t="n">
+      <c r="D12" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="19" t="n">
         <v>2.9</v>
       </c>
-      <c r="G12" s="20" t="n">
+      <c r="G12" s="19" t="n">
         <v>73.2</v>
       </c>
-      <c r="H12" s="20" t="n">
+      <c r="H12" s="19" t="n">
         <v>90</v>
       </c>
-      <c r="I12" s="20" t="n">
+      <c r="I12" s="19" t="n">
         <v>4</v>
       </c>
-      <c r="J12" s="14">
+      <c r="J12" s="13">
         <f>Img_Class_outs!E7 - F12</f>
         <v/>
       </c>
-      <c r="K12" s="14">
+      <c r="K12" s="13">
         <f>J12/F12 * 100</f>
         <v/>
       </c>
     </row>
-    <row r="13" ht="29.25" customHeight="1" s="15">
-      <c r="A13" s="18" t="inlineStr">
+    <row r="13" ht="29.25" customHeight="1" s="14">
+      <c r="A13" s="17" t="inlineStr">
         <is>
           <t>MobileNet V2 (TF_ver_2.0)</t>
         </is>
       </c>
-      <c r="B13" s="19" t="inlineStr">
+      <c r="B13" s="18" t="inlineStr">
         <is>
           <t>1,000 objects
 ILSVRC2012</t>
         </is>
       </c>
-      <c r="C13" s="20" t="inlineStr">
+      <c r="C13" s="19" t="inlineStr">
         <is>
           <t>224x224x3</t>
         </is>
       </c>
-      <c r="D13" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="E13" s="20" t="n">
+      <c r="D13" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="19" t="n">
         <v>2</v>
       </c>
-      <c r="F13" s="20" t="n">
+      <c r="F13" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="G13" s="20" t="n">
+      <c r="G13" s="19" t="n">
         <v>73.2</v>
       </c>
-      <c r="H13" s="20" t="n">
+      <c r="H13" s="19" t="n">
         <v>91.8</v>
       </c>
-      <c r="I13" s="20" t="n">
+      <c r="I13" s="19" t="n">
         <v>4.1</v>
       </c>
-      <c r="J13" s="14">
+      <c r="J13" s="13">
         <f>Img_Class_outs!E4-F13</f>
         <v/>
       </c>
-      <c r="K13" s="14">
+      <c r="K13" s="13">
         <f>J13/F13 * 100</f>
         <v/>
       </c>
     </row>
-    <row r="14" ht="23.05" customHeight="1" s="15">
-      <c r="A14" s="18" t="inlineStr">
+    <row r="14" ht="22.5" customHeight="1" s="14">
+      <c r="A14" s="17" t="inlineStr">
         <is>
           <t>MobileNet V3</t>
         </is>
       </c>
-      <c r="B14" s="19" t="inlineStr">
+      <c r="B14" s="18" t="inlineStr">
         <is>
           <t>1,000 objects
 ILSVRC2012</t>
         </is>
       </c>
-      <c r="C14" s="20" t="inlineStr">
+      <c r="C14" s="19" t="inlineStr">
         <is>
           <t>224x224x3</t>
         </is>
       </c>
-      <c r="D14" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="E14" s="20" t="n">
+      <c r="D14" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="19" t="n">
         <v>2</v>
       </c>
-      <c r="F14" s="20" t="n">
+      <c r="F14" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="G14" s="20" t="n">
+      <c r="G14" s="19" t="n">
         <v>77.5</v>
       </c>
-      <c r="H14" s="20" t="n">
+      <c r="H14" s="19" t="n">
         <v>93.59999999999999</v>
       </c>
-      <c r="I14" s="20" t="n">
+      <c r="I14" s="19" t="n">
         <v>4.9</v>
       </c>
-      <c r="J14" s="14">
+      <c r="J14" s="13">
         <f>Img_Class_outs!E6-F14</f>
         <v/>
       </c>
-      <c r="K14" s="14">
+      <c r="K14" s="13">
         <f>J14/F14 * 100</f>
         <v/>
       </c>
@@ -1333,321 +1236,321 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="23" t="inlineStr">
+      <c r="A1" s="20" t="inlineStr">
         <is>
           <t>Model name</t>
         </is>
       </c>
-      <c r="B1" s="23" t="inlineStr">
+      <c r="B1" s="20" t="inlineStr">
         <is>
           <t>Latency (ms)</t>
         </is>
       </c>
-      <c r="C1" s="23" t="inlineStr">
+      <c r="C1" s="20" t="inlineStr">
         <is>
           <t>Top-1 Accuracy</t>
         </is>
       </c>
-      <c r="D1" s="23" t="inlineStr">
+      <c r="D1" s="20" t="inlineStr">
         <is>
           <t>Top-5 Accuracy</t>
         </is>
       </c>
-      <c r="E1" s="23" t="inlineStr">
+      <c r="E1" s="20" t="inlineStr">
         <is>
           <t>Measured Inference Time (ms)</t>
         </is>
       </c>
-      <c r="F1" s="23" t="inlineStr">
+      <c r="F1" s="20" t="inlineStr">
         <is>
           <t>Parameter Count (M)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="14" t="inlineStr">
+      <c r="A2" s="13" t="inlineStr">
         <is>
           <t>MobileNet V1 (0.25)</t>
         </is>
       </c>
-      <c r="B2" s="14" t="n">
+      <c r="B2" s="13" t="n">
         <v>0.9</v>
       </c>
-      <c r="C2" s="14" t="n">
+      <c r="C2" s="13" t="n">
         <v>40.8</v>
       </c>
-      <c r="D2" s="14" t="n">
+      <c r="D2" s="13" t="n">
         <v>95.09999999999999</v>
       </c>
-      <c r="E2" s="14" t="n">
+      <c r="E2" s="13" t="n">
         <v>4.273343636746742</v>
       </c>
-      <c r="F2" s="14" t="n">
+      <c r="F2" s="13" t="n">
         <v>0.467595</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="14" t="inlineStr">
+      <c r="A3" s="13" t="inlineStr">
         <is>
           <t>MobileNet V1 (0.50)</t>
         </is>
       </c>
-      <c r="B3" s="14" t="n">
+      <c r="B3" s="13" t="n">
         <v>1.4</v>
       </c>
-      <c r="C3" s="14" t="n">
+      <c r="C3" s="13" t="n">
         <v>63.7</v>
       </c>
-      <c r="D3" s="14" t="n">
+      <c r="D3" s="13" t="n">
         <v>94.5</v>
       </c>
-      <c r="E3" s="14" t="n">
+      <c r="E3" s="13" t="n">
         <v>5.741725413576729</v>
       </c>
-      <c r="F3" s="14" t="n">
+      <c r="F3" s="13" t="n">
+        <v>1.326635</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="13" t="inlineStr">
+        <is>
+          <t>MobileNet V1 (1.0)</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="C4" s="13" t="n">
+        <v>69.5</v>
+      </c>
+      <c r="D4" s="13" t="n">
+        <v>94.7</v>
+      </c>
+      <c r="E4" s="13" t="n">
+        <v>6.408314722753338</v>
+      </c>
+      <c r="F4" s="13" t="n">
         <v>4.899478</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="14" t="inlineStr">
-        <is>
-          <t>MobileNet V1 (1.0)</t>
-        </is>
-      </c>
-      <c r="B4" s="14" t="n">
+    <row r="5">
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>MobileNet V1 (.75)</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="C5" s="13" t="n">
+        <v>67.2</v>
+      </c>
+      <c r="D5" s="13" t="n">
+        <v>92</v>
+      </c>
+      <c r="E5" s="13" t="n">
+        <v>6.413245242038233</v>
+      </c>
+      <c r="F5" s="13" t="n">
+        <v>2.578123</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t>MobileNet V2</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="C6" s="13" t="n">
+        <v>73.2</v>
+      </c>
+      <c r="D6" s="13" t="n">
+        <v>93.2</v>
+      </c>
+      <c r="E6" s="13" t="n">
+        <v>7.892005935786992</v>
+      </c>
+      <c r="F6" s="13" t="n">
+        <v>3.489099</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t>MobileNet V2 (TF_ver_2.0)</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="C7" s="13" t="n">
+        <v>73.2</v>
+      </c>
+      <c r="D7" s="13" t="n">
+        <v>67.2</v>
+      </c>
+      <c r="E7" s="13" t="n">
+        <v>8.365876630525435</v>
+      </c>
+      <c r="F7" s="13" t="n">
+        <v>3.489101</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="13" t="inlineStr">
+        <is>
+          <t>MobileNet V1 (TF_ver_2.0)</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="n">
         <v>2.8</v>
       </c>
-      <c r="C4" s="14" t="n">
+      <c r="C8" s="13" t="n">
         <v>69.5</v>
       </c>
-      <c r="D4" s="14" t="n">
-        <v>94.7</v>
-      </c>
-      <c r="E4" s="14" t="n">
-        <v>6.408314722753338</v>
-      </c>
-      <c r="F4" s="14" t="n">
-        <v>1.326635</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="14" t="inlineStr">
-        <is>
-          <t>MobileNet V1 (.75)</t>
-        </is>
-      </c>
-      <c r="B5" s="14" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="C5" s="14" t="n">
-        <v>67.2</v>
-      </c>
-      <c r="D5" s="14" t="n">
-        <v>92</v>
-      </c>
-      <c r="E5" s="14" t="n">
-        <v>6.413245242038233</v>
-      </c>
-      <c r="F5" s="14" t="n">
+      <c r="D8" s="13" t="n">
+        <v>83.40000000000001</v>
+      </c>
+      <c r="E8" s="13" t="n">
+        <v>8.588968593350385</v>
+      </c>
+      <c r="F8" s="13" t="n">
         <v>4.222061</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="14" t="inlineStr">
-        <is>
-          <t>MobileNet V2</t>
-        </is>
-      </c>
-      <c r="B6" s="14" t="n">
-        <v>2.9</v>
-      </c>
-      <c r="C6" s="14" t="n">
-        <v>73.2</v>
-      </c>
-      <c r="D6" s="14" t="n">
-        <v>93.2</v>
-      </c>
-      <c r="E6" s="14" t="n">
-        <v>7.892005935786992</v>
-      </c>
-      <c r="F6" s="14" t="n">
+    <row r="9">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>MobileNet V3</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="C9" s="13" t="n">
+        <v>77.5</v>
+      </c>
+      <c r="D9" s="13" t="n">
+        <v>88.09999999999999</v>
+      </c>
+      <c r="E9" s="13" t="n">
+        <v>8.700641511226253</v>
+      </c>
+      <c r="F9" s="13" t="n">
+        <v>4.073277</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="13" t="inlineStr">
+        <is>
+          <t>EfficientNet-EdgeTpu (S)</t>
+        </is>
+      </c>
+      <c r="B10" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="C10" s="13" t="n">
+        <v>78.90000000000001</v>
+      </c>
+      <c r="D10" s="13" t="n">
+        <v>90.59999999999999</v>
+      </c>
+      <c r="E10" s="13" t="n">
+        <v>9.05769085895118</v>
+      </c>
+      <c r="F10" s="13" t="n">
+        <v>5.413955</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>Inception V1</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="C11" s="13" t="n">
+        <v>71.90000000000001</v>
+      </c>
+      <c r="D11" s="13" t="n">
+        <v>89.8</v>
+      </c>
+      <c r="E11" s="13" t="n">
+        <v>15.37397241960187</v>
+      </c>
+      <c r="F11" s="13" t="n">
+        <v>6.618651</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>EfficientNet-EdgeTpu (M)</t>
+        </is>
+      </c>
+      <c r="B12" s="13" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="C12" s="13" t="n">
+        <v>80.09999999999999</v>
+      </c>
+      <c r="D12" s="13" t="n">
+        <v>90</v>
+      </c>
+      <c r="E12" s="13" t="n">
+        <v>26.50050885333329</v>
+      </c>
+      <c r="F12" s="13" t="n">
         <v>6.866875</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="14" t="inlineStr">
-        <is>
-          <t>MobileNet V2 (TF_ver_2.0)</t>
-        </is>
-      </c>
-      <c r="B7" s="14" t="n">
-        <v>3</v>
-      </c>
-      <c r="C7" s="14" t="n">
-        <v>73.2</v>
-      </c>
-      <c r="D7" s="14" t="n">
-        <v>67.2</v>
-      </c>
-      <c r="E7" s="14" t="n">
-        <v>8.365876630525435</v>
-      </c>
-      <c r="F7" s="14" t="n">
-        <v>5.413955</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="14" t="inlineStr">
-        <is>
-          <t>MobileNet V1 (TF_ver_2.0)</t>
-        </is>
-      </c>
-      <c r="B8" s="14" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="C8" s="14" t="n">
-        <v>69.5</v>
-      </c>
-      <c r="D8" s="14" t="n">
-        <v>83.40000000000001</v>
-      </c>
-      <c r="E8" s="14" t="n">
-        <v>8.588968593350385</v>
-      </c>
-      <c r="F8" s="14" t="n">
-        <v>2.578123</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="14" t="inlineStr">
-        <is>
-          <t>MobileNet V3</t>
-        </is>
-      </c>
-      <c r="B9" s="14" t="n">
-        <v>3</v>
-      </c>
-      <c r="C9" s="14" t="n">
-        <v>77.5</v>
-      </c>
-      <c r="D9" s="14" t="n">
-        <v>88.09999999999999</v>
-      </c>
-      <c r="E9" s="14" t="n">
-        <v>8.700641511226253</v>
-      </c>
-      <c r="F9" s="14" t="n">
+    <row r="13">
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>EfficientNet-EdgeTpu (L)</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="n">
+        <v>21.3</v>
+      </c>
+      <c r="C13" s="13" t="n">
+        <v>81.2</v>
+      </c>
+      <c r="D13" s="13" t="n">
+        <v>91.8</v>
+      </c>
+      <c r="E13" s="13" t="n">
+        <v>102.4790272164949</v>
+      </c>
+      <c r="F13" s="13" t="n">
         <v>10.545147</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="14" t="inlineStr">
-        <is>
-          <t>EfficientNet-EdgeTpu (S)</t>
-        </is>
-      </c>
-      <c r="B10" s="14" t="n">
-        <v>5</v>
-      </c>
-      <c r="C10" s="14" t="n">
-        <v>78.90000000000001</v>
-      </c>
-      <c r="D10" s="14" t="n">
-        <v>90.59999999999999</v>
-      </c>
-      <c r="E10" s="14" t="n">
-        <v>9.05769085895118</v>
-      </c>
-      <c r="F10" s="14" t="n">
-        <v>3.489101</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="14" t="inlineStr">
-        <is>
-          <t>Inception V1</t>
-        </is>
-      </c>
-      <c r="B11" s="14" t="n">
-        <v>3.4</v>
-      </c>
-      <c r="C11" s="14" t="n">
-        <v>71.90000000000001</v>
-      </c>
-      <c r="D11" s="14" t="n">
-        <v>89.8</v>
-      </c>
-      <c r="E11" s="14" t="n">
-        <v>15.37397241960187</v>
-      </c>
-      <c r="F11" s="14" t="n">
-        <v>3.489099</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="14" t="inlineStr">
-        <is>
-          <t>EfficientNet-EdgeTpu (M)</t>
-        </is>
-      </c>
-      <c r="B12" s="14" t="n">
-        <v>7.3</v>
-      </c>
-      <c r="C12" s="14" t="n">
-        <v>80.09999999999999</v>
-      </c>
-      <c r="D12" s="14" t="n">
-        <v>90</v>
-      </c>
-      <c r="E12" s="14" t="n">
-        <v>26.50050885333329</v>
-      </c>
-      <c r="F12" s="14" t="n">
-        <v>6.618651</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="14" t="inlineStr">
-        <is>
-          <t>EfficientNet-EdgeTpu (L)</t>
-        </is>
-      </c>
-      <c r="B13" s="14" t="n">
-        <v>21.3</v>
-      </c>
-      <c r="C13" s="14" t="n">
-        <v>81.2</v>
-      </c>
-      <c r="D13" s="14" t="n">
-        <v>91.8</v>
-      </c>
-      <c r="E13" s="14" t="n">
-        <v>102.4790272164949</v>
-      </c>
-      <c r="F13" s="14" t="n">
+    <row r="14">
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t>Inception V3</t>
+        </is>
+      </c>
+      <c r="B14" s="13" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="C14" s="13" t="n">
+        <v>75.40000000000001</v>
+      </c>
+      <c r="D14" s="13" t="n">
+        <v>93.59999999999999</v>
+      </c>
+      <c r="E14" s="13" t="n">
+        <v>118.5258274698795</v>
+      </c>
+      <c r="F14" s="13" t="n">
         <v>11.179387</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="14" t="inlineStr">
-        <is>
-          <t>Inception V3</t>
-        </is>
-      </c>
-      <c r="B14" s="14" t="n">
-        <v>13.4</v>
-      </c>
-      <c r="C14" s="14" t="n">
-        <v>75.40000000000001</v>
-      </c>
-      <c r="D14" s="14" t="n">
-        <v>93.59999999999999</v>
-      </c>
-      <c r="E14" s="14" t="n">
-        <v>118.5258274698795</v>
-      </c>
-      <c r="F14" s="14" t="n">
-        <v>4.073277</v>
       </c>
     </row>
   </sheetData>
@@ -1664,196 +1567,196 @@
   <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="20.29" customWidth="1" style="14" min="1" max="1"/>
-    <col width="16.57" customWidth="1" style="14" min="2" max="2"/>
-    <col width="17" customWidth="1" style="14" min="3" max="3"/>
-    <col width="13.29" customWidth="1" style="14" min="4" max="4"/>
-    <col width="12.29" customWidth="1" style="14" min="5" max="5"/>
+    <col width="20.29" customWidth="1" style="13" min="1" max="1"/>
+    <col width="16.57" customWidth="1" style="13" min="2" max="2"/>
+    <col width="17" customWidth="1" style="13" min="3" max="3"/>
+    <col width="13.3" customWidth="1" style="13" min="4" max="4"/>
+    <col width="12.29" customWidth="1" style="13" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1" s="15">
-      <c r="A1" s="14" t="inlineStr">
+    <row r="1" ht="15" customHeight="1" s="14">
+      <c r="A1" s="13" t="inlineStr">
         <is>
           <t>Model Name</t>
         </is>
       </c>
-      <c r="D1" s="14" t="inlineStr">
+      <c r="D1" s="13" t="inlineStr">
         <is>
           <t>Latency (ms)</t>
         </is>
       </c>
-      <c r="E1" s="14" t="inlineStr">
+      <c r="E1" s="13" t="inlineStr">
         <is>
           <t>mAP</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="29.25" customHeight="1" s="15">
-      <c r="A2" s="18" t="inlineStr">
+    <row r="2" ht="29.25" customHeight="1" s="14">
+      <c r="A2" s="17" t="inlineStr">
         <is>
           <t>SSD MobileNet V1</t>
         </is>
       </c>
-      <c r="B2" s="19" t="inlineStr">
+      <c r="B2" s="18" t="inlineStr">
         <is>
           <t>90 objects
 COCO</t>
         </is>
       </c>
-      <c r="C2" s="20" t="inlineStr">
+      <c r="C2" s="19" t="inlineStr">
         <is>
           <t>300x300x3</t>
         </is>
       </c>
-      <c r="D2" s="20" t="n">
+      <c r="D2" s="19" t="n">
         <v>6.5</v>
       </c>
-      <c r="E2" s="20" t="n">
+      <c r="E2" s="19" t="n">
         <v>21.5</v>
       </c>
-      <c r="F2" s="20" t="inlineStr">
+      <c r="F2" s="19" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="G2" s="20" t="inlineStr">
+      <c r="G2" s="19" t="inlineStr">
         <is>
           <t>7.0 MB</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="36" customHeight="1" s="15">
-      <c r="A3" s="18" t="inlineStr">
+    <row r="3" ht="36" customHeight="1" s="14">
+      <c r="A3" s="17" t="inlineStr">
         <is>
           <t>SSD MobileNet V2(TF1)</t>
         </is>
       </c>
-      <c r="B3" s="19" t="inlineStr">
+      <c r="B3" s="18" t="inlineStr">
         <is>
           <t>90 objects
 COCO</t>
         </is>
       </c>
-      <c r="C3" s="20" t="inlineStr">
+      <c r="C3" s="19" t="inlineStr">
         <is>
           <t>300x300x3</t>
         </is>
       </c>
-      <c r="D3" s="20" t="n">
+      <c r="D3" s="19" t="n">
         <v>7.3</v>
       </c>
-      <c r="E3" s="20" t="n">
+      <c r="E3" s="19" t="n">
         <v>25.6</v>
       </c>
-      <c r="F3" s="20" t="inlineStr">
+      <c r="F3" s="19" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="G3" s="20" t="inlineStr">
+      <c r="G3" s="19" t="inlineStr">
         <is>
           <t>6.6 MB</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="36" customHeight="1" s="15">
-      <c r="A4" s="18" t="inlineStr">
+    <row r="4" ht="36" customHeight="1" s="14">
+      <c r="A4" s="17" t="inlineStr">
         <is>
           <t>SSD MobileNet V2 (TF2)</t>
         </is>
       </c>
-      <c r="B4" s="19" t="inlineStr">
+      <c r="B4" s="18" t="inlineStr">
         <is>
           <t>90 objects
 COCO</t>
         </is>
       </c>
-      <c r="C4" s="20" t="inlineStr">
+      <c r="C4" s="19" t="inlineStr">
         <is>
           <t>300x300x3</t>
         </is>
       </c>
-      <c r="D4" s="20" t="n">
+      <c r="D4" s="19" t="n">
         <v>7.6</v>
       </c>
-      <c r="E4" s="20" t="n">
+      <c r="E4" s="19" t="n">
         <v>22.4</v>
       </c>
-      <c r="F4" s="20" t="inlineStr">
+      <c r="F4" s="19" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="G4" s="20" t="inlineStr">
+      <c r="G4" s="19" t="inlineStr">
         <is>
           <t>6.7 MB</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="17.25" customHeight="1" s="15">
-      <c r="A5" s="18" t="inlineStr">
+    <row r="5" ht="17.25" customHeight="1" s="14">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>SSD MobileNet V2</t>
         </is>
       </c>
-      <c r="B5" s="18" t="inlineStr">
+      <c r="B5" s="17" t="inlineStr">
         <is>
           <t>Faces</t>
         </is>
       </c>
-      <c r="C5" s="20" t="inlineStr">
+      <c r="C5" s="19" t="inlineStr">
         <is>
           <t>320x320x3</t>
         </is>
       </c>
-      <c r="D5" s="20" t="n">
+      <c r="D5" s="19" t="n">
         <v>5.2</v>
       </c>
-      <c r="E5" s="20" t="inlineStr">
+      <c r="E5" s="19" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="F5" s="20" t="inlineStr">
+      <c r="F5" s="19" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="G5" s="20" t="inlineStr">
+      <c r="G5" s="19" t="inlineStr">
         <is>
           <t>6.7 MB</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="29.25" customHeight="1" s="15">
-      <c r="A6" s="18" t="inlineStr">
+    <row r="6" ht="29.25" customHeight="1" s="14">
+      <c r="A6" s="17" t="inlineStr">
         <is>
           <t>SSDLite MobileDet</t>
         </is>
       </c>
-      <c r="B6" s="19" t="inlineStr">
+      <c r="B6" s="18" t="inlineStr">
         <is>
           <t>90 objects
 COCO</t>
         </is>
       </c>
-      <c r="C6" s="20" t="inlineStr">
+      <c r="C6" s="19" t="inlineStr">
         <is>
           <t>320x320x3</t>
         </is>
       </c>
-      <c r="D6" s="20" t="n">
+      <c r="D6" s="19" t="n">
         <v>9.1</v>
       </c>
-      <c r="E6" s="20" t="n">
+      <c r="E6" s="19" t="n">
         <v>32.9</v>
       </c>
-      <c r="F6" s="20" t="inlineStr">
+      <c r="F6" s="19" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="G6" s="20" t="inlineStr">
+      <c r="G6" s="19" t="inlineStr">
         <is>
           <t>5.1 MB</t>
         </is>
@@ -1881,167 +1784,167 @@
   <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="29.29" customWidth="1" style="14" min="1" max="1"/>
-    <col width="21.43" customWidth="1" style="14" min="2" max="2"/>
-    <col width="16.86" customWidth="1" style="14" min="3" max="4"/>
-    <col width="14.71" customWidth="1" style="14" min="8" max="8"/>
-    <col width="12" customWidth="1" style="14" min="10" max="10"/>
+    <col width="29.3" customWidth="1" style="13" min="1" max="1"/>
+    <col width="21.43" customWidth="1" style="13" min="2" max="2"/>
+    <col width="16.86" customWidth="1" style="13" min="3" max="4"/>
+    <col width="14.7" customWidth="1" style="13" min="8" max="8"/>
+    <col width="12" customWidth="1" style="13" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1" s="15">
-      <c r="A1" s="14" t="inlineStr">
+    <row r="1" ht="15" customHeight="1" s="14">
+      <c r="A1" s="13" t="inlineStr">
         <is>
           <t>Model Name</t>
         </is>
       </c>
-      <c r="C1" s="14" t="inlineStr">
+      <c r="C1" s="13" t="inlineStr">
         <is>
           <t>Input Size</t>
         </is>
       </c>
-      <c r="D1" s="14" t="inlineStr">
+      <c r="D1" s="13" t="inlineStr">
         <is>
           <t>Params (flatbuffers)</t>
         </is>
       </c>
-      <c r="H1" s="14" t="inlineStr">
+      <c r="H1" s="13" t="inlineStr">
         <is>
           <t>Latency (ms)</t>
         </is>
       </c>
-      <c r="J1" s="14" t="inlineStr">
+      <c r="J1" s="13" t="inlineStr">
         <is>
           <t>Model Size</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="29.25" customHeight="1" s="15">
-      <c r="A2" s="18" t="inlineStr">
+    <row r="2" ht="29.25" customHeight="1" s="14">
+      <c r="A2" s="17" t="inlineStr">
         <is>
           <t>U-Net MobileNet v2</t>
         </is>
       </c>
-      <c r="B2" s="19" t="inlineStr">
+      <c r="B2" s="18" t="inlineStr">
         <is>
           <t>37 pets
 Oxford-IIIT pets</t>
         </is>
       </c>
-      <c r="C2" s="20" t="inlineStr">
+      <c r="C2" s="19" t="inlineStr">
         <is>
           <t>128x128x3</t>
         </is>
       </c>
-      <c r="D2" s="20" t="n"/>
-      <c r="E2" s="20" t="inlineStr">
+      <c r="D2" s="19" t="n"/>
+      <c r="E2" s="19" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="F2" s="20" t="inlineStr">
+      <c r="F2" s="19" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="G2" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="H2" s="20" t="n">
+      <c r="G2" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" s="19" t="n">
         <v>2.7</v>
       </c>
-      <c r="I2" s="20" t="inlineStr">
+      <c r="I2" s="19" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="J2" s="20" t="inlineStr">
+      <c r="J2" s="19" t="inlineStr">
         <is>
           <t>7.2 MB</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="29.25" customHeight="1" s="15">
-      <c r="A3" s="18" t="inlineStr">
+    <row r="3" ht="29.25" customHeight="1" s="14">
+      <c r="A3" s="17" t="inlineStr">
         <is>
           <t>U-Net MobileNet v2</t>
         </is>
       </c>
-      <c r="B3" s="19" t="inlineStr">
+      <c r="B3" s="18" t="inlineStr">
         <is>
           <t>37 pets
 Oxford-IIIT pets</t>
         </is>
       </c>
-      <c r="C3" s="20" t="inlineStr">
+      <c r="C3" s="19" t="inlineStr">
         <is>
           <t>256x256x3</t>
         </is>
       </c>
-      <c r="D3" s="20" t="n"/>
-      <c r="E3" s="20" t="inlineStr">
+      <c r="D3" s="19" t="n"/>
+      <c r="E3" s="19" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="F3" s="20" t="inlineStr">
+      <c r="F3" s="19" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="G3" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="H3" s="20" t="n">
+      <c r="G3" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" s="19" t="n">
         <v>29</v>
       </c>
-      <c r="I3" s="20" t="inlineStr">
+      <c r="I3" s="19" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="J3" s="20" t="inlineStr">
+      <c r="J3" s="19" t="inlineStr">
         <is>
           <t>7.3 MB</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="17.25" customHeight="1" s="15">
-      <c r="A4" s="24" t="inlineStr">
+    <row r="4" ht="17.25" customHeight="1" s="14">
+      <c r="A4" s="21" t="inlineStr">
         <is>
           <t>MobileNet v1 BodyPix</t>
         </is>
       </c>
-      <c r="B4" s="24" t="inlineStr">
+      <c r="B4" s="21" t="inlineStr">
         <is>
           <t>24 body parts</t>
         </is>
       </c>
-      <c r="C4" s="25" t="inlineStr">
+      <c r="C4" s="22" t="inlineStr">
         <is>
           <t>324x324x3</t>
         </is>
       </c>
-      <c r="D4" s="25" t="n"/>
-      <c r="E4" s="25" t="n">
+      <c r="D4" s="22" t="n"/>
+      <c r="E4" s="22" t="n">
         <v>0.75</v>
       </c>
-      <c r="F4" s="25" t="n">
+      <c r="F4" s="22" t="n">
         <v>16</v>
       </c>
-      <c r="G4" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="H4" s="25" t="inlineStr">
+      <c r="G4" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="H4" s="22" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="I4" s="25" t="inlineStr">
+      <c r="I4" s="22" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="J4" s="25" t="inlineStr">
+      <c r="J4" s="22" t="inlineStr">
         <is>
           <t>1.6 MB</t>
         </is>
@@ -2067,407 +1970,407 @@
   <dimension ref="A1:J10"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="29.29" customWidth="1" style="14" min="1" max="1"/>
-    <col width="21.43" customWidth="1" style="14" min="2" max="2"/>
-    <col width="16.86" customWidth="1" style="14" min="3" max="4"/>
-    <col width="14.71" customWidth="1" style="14" min="8" max="8"/>
-    <col width="12" customWidth="1" style="14" min="10" max="10"/>
+    <col width="29.3" customWidth="1" style="13" min="1" max="1"/>
+    <col width="21.43" customWidth="1" style="13" min="2" max="2"/>
+    <col width="16.86" customWidth="1" style="13" min="3" max="4"/>
+    <col width="14.7" customWidth="1" style="13" min="8" max="8"/>
+    <col width="12" customWidth="1" style="13" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1" s="15">
-      <c r="A1" s="14" t="inlineStr">
+    <row r="1" ht="15" customHeight="1" s="14">
+      <c r="A1" s="13" t="inlineStr">
         <is>
           <t>Model Name</t>
         </is>
       </c>
-      <c r="C1" s="14" t="inlineStr">
+      <c r="C1" s="13" t="inlineStr">
         <is>
           <t>Input Size</t>
         </is>
       </c>
-      <c r="D1" s="14" t="inlineStr">
+      <c r="D1" s="13" t="inlineStr">
         <is>
           <t>Params (flatbuffers)</t>
         </is>
       </c>
-      <c r="H1" s="14" t="inlineStr">
+      <c r="H1" s="13" t="inlineStr">
         <is>
           <t>Latency (ms)</t>
         </is>
       </c>
-      <c r="J1" s="14" t="inlineStr">
+      <c r="J1" s="13" t="inlineStr">
         <is>
           <t>Model Size</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="29.25" customHeight="1" s="15">
-      <c r="A2" s="18" t="inlineStr">
+    <row r="2" ht="29.25" customHeight="1" s="14">
+      <c r="A2" s="17" t="inlineStr">
         <is>
           <t>U-Net MobileNet v2</t>
         </is>
       </c>
-      <c r="B2" s="19" t="inlineStr">
+      <c r="B2" s="18" t="inlineStr">
         <is>
           <t>37 pets
 Oxford-IIIT pets</t>
         </is>
       </c>
-      <c r="C2" s="20" t="inlineStr">
+      <c r="C2" s="19" t="inlineStr">
         <is>
           <t>128x128x3</t>
         </is>
       </c>
-      <c r="D2" s="20" t="n"/>
-      <c r="E2" s="20" t="inlineStr">
+      <c r="D2" s="19" t="n"/>
+      <c r="E2" s="19" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="F2" s="20" t="inlineStr">
+      <c r="F2" s="19" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="G2" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="H2" s="20" t="n">
+      <c r="G2" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" s="19" t="n">
         <v>2.7</v>
       </c>
-      <c r="I2" s="20" t="inlineStr">
+      <c r="I2" s="19" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="J2" s="20" t="inlineStr">
+      <c r="J2" s="19" t="inlineStr">
         <is>
           <t>7.2 MB</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="29.25" customHeight="1" s="15">
-      <c r="A3" s="18" t="inlineStr">
+    <row r="3" ht="29.25" customHeight="1" s="14">
+      <c r="A3" s="17" t="inlineStr">
         <is>
           <t>U-Net MobileNet v2</t>
         </is>
       </c>
-      <c r="B3" s="19" t="inlineStr">
+      <c r="B3" s="18" t="inlineStr">
         <is>
           <t>37 pets
 Oxford-IIIT pets</t>
         </is>
       </c>
-      <c r="C3" s="20" t="inlineStr">
+      <c r="C3" s="19" t="inlineStr">
         <is>
           <t>256x256x3</t>
         </is>
       </c>
-      <c r="D3" s="20" t="n"/>
-      <c r="E3" s="20" t="inlineStr">
+      <c r="D3" s="19" t="n"/>
+      <c r="E3" s="19" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="F3" s="20" t="inlineStr">
+      <c r="F3" s="19" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="G3" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="H3" s="20" t="n">
+      <c r="G3" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" s="19" t="n">
         <v>29</v>
       </c>
-      <c r="I3" s="20" t="inlineStr">
+      <c r="I3" s="19" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="J3" s="20" t="inlineStr">
+      <c r="J3" s="19" t="inlineStr">
         <is>
           <t>7.3 MB</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="17.25" customHeight="1" s="15">
-      <c r="A4" s="24" t="inlineStr">
+    <row r="4" ht="17.25" customHeight="1" s="14">
+      <c r="A4" s="21" t="inlineStr">
         <is>
           <t>MobileNet v1 BodyPix</t>
         </is>
       </c>
-      <c r="B4" s="24" t="inlineStr">
+      <c r="B4" s="21" t="inlineStr">
         <is>
           <t>24 body parts</t>
         </is>
       </c>
-      <c r="C4" s="25" t="inlineStr">
+      <c r="C4" s="22" t="inlineStr">
         <is>
           <t>324x324x3</t>
         </is>
       </c>
-      <c r="D4" s="25" t="n"/>
-      <c r="E4" s="25" t="n">
+      <c r="D4" s="22" t="n"/>
+      <c r="E4" s="22" t="n">
         <v>0.75</v>
       </c>
-      <c r="F4" s="25" t="n">
+      <c r="F4" s="22" t="n">
         <v>16</v>
       </c>
-      <c r="G4" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="H4" s="25" t="inlineStr">
+      <c r="G4" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="H4" s="22" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="I4" s="25" t="inlineStr">
+      <c r="I4" s="22" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="J4" s="25" t="inlineStr">
+      <c r="J4" s="22" t="inlineStr">
         <is>
           <t>1.6 MB</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="17.25" customHeight="1" s="15">
-      <c r="A5" s="18" t="inlineStr">
+    <row r="5" ht="17.25" customHeight="1" s="14">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>MobileNet v1 BodyPix</t>
         </is>
       </c>
-      <c r="B5" s="18" t="inlineStr">
+      <c r="B5" s="17" t="inlineStr">
         <is>
           <t>24 body parts</t>
         </is>
       </c>
-      <c r="C5" s="20" t="inlineStr">
+      <c r="C5" s="19" t="inlineStr">
         <is>
           <t>352x480x3</t>
         </is>
       </c>
-      <c r="D5" s="20" t="n"/>
-      <c r="E5" s="20" t="n">
+      <c r="D5" s="19" t="n"/>
+      <c r="E5" s="19" t="n">
         <v>0.75</v>
       </c>
-      <c r="F5" s="20" t="n">
+      <c r="F5" s="19" t="n">
         <v>16</v>
       </c>
-      <c r="G5" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="H5" s="20" t="n">
+      <c r="G5" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" s="19" t="n">
         <v>6.9</v>
       </c>
-      <c r="I5" s="20" t="inlineStr">
+      <c r="I5" s="19" t="inlineStr">
         <is>
           <t>Yes*</t>
         </is>
       </c>
-      <c r="J5" s="20" t="inlineStr">
+      <c r="J5" s="19" t="inlineStr">
         <is>
           <t>1.6 MB</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="17.25" customHeight="1" s="15">
-      <c r="A6" s="18" t="inlineStr">
+    <row r="6" ht="17.25" customHeight="1" s="14">
+      <c r="A6" s="17" t="inlineStr">
         <is>
           <t>MobileNet v1 BodyPix</t>
         </is>
       </c>
-      <c r="B6" s="18" t="inlineStr">
+      <c r="B6" s="17" t="inlineStr">
         <is>
           <t>24 body parts</t>
         </is>
       </c>
-      <c r="C6" s="20" t="inlineStr">
+      <c r="C6" s="19" t="inlineStr">
         <is>
           <t>512x512x3</t>
         </is>
       </c>
-      <c r="D6" s="20" t="n"/>
-      <c r="E6" s="20" t="n">
+      <c r="D6" s="19" t="n"/>
+      <c r="E6" s="19" t="n">
         <v>0.75</v>
       </c>
-      <c r="F6" s="20" t="n">
+      <c r="F6" s="19" t="n">
         <v>16</v>
       </c>
-      <c r="G6" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="H6" s="20" t="n">
+      <c r="G6" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" s="19" t="n">
         <v>10.7</v>
       </c>
-      <c r="I6" s="20" t="inlineStr">
+      <c r="I6" s="19" t="inlineStr">
         <is>
           <t>Yes*</t>
         </is>
       </c>
-      <c r="J6" s="20" t="inlineStr">
+      <c r="J6" s="19" t="inlineStr">
         <is>
           <t>1.7 MB</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="17.25" customHeight="1" s="15">
-      <c r="A7" s="18" t="inlineStr">
+    <row r="7" ht="17.25" customHeight="1" s="14">
+      <c r="A7" s="17" t="inlineStr">
         <is>
           <t>MobileNet v1 BodyPix</t>
         </is>
       </c>
-      <c r="B7" s="18" t="inlineStr">
+      <c r="B7" s="17" t="inlineStr">
         <is>
           <t>24 body parts</t>
         </is>
       </c>
-      <c r="C7" s="20" t="inlineStr">
+      <c r="C7" s="19" t="inlineStr">
         <is>
           <t>480x640x3</t>
         </is>
       </c>
-      <c r="D7" s="20" t="n"/>
-      <c r="E7" s="20" t="n">
+      <c r="D7" s="19" t="n"/>
+      <c r="E7" s="19" t="n">
         <v>0.75</v>
       </c>
-      <c r="F7" s="20" t="n">
+      <c r="F7" s="19" t="n">
         <v>16</v>
       </c>
-      <c r="G7" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="H7" s="20" t="n">
+      <c r="G7" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" s="19" t="n">
         <v>12.3</v>
       </c>
-      <c r="I7" s="20" t="inlineStr">
+      <c r="I7" s="19" t="inlineStr">
         <is>
           <t>Yes*</t>
         </is>
       </c>
-      <c r="J7" s="20" t="inlineStr">
+      <c r="J7" s="19" t="inlineStr">
         <is>
           <t>1.8 MB</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="17.25" customHeight="1" s="15">
-      <c r="A8" s="18" t="inlineStr">
+    <row r="8" ht="17.25" customHeight="1" s="14">
+      <c r="A8" s="17" t="inlineStr">
         <is>
           <t>MobileNet v1 BodyPix</t>
         </is>
       </c>
-      <c r="B8" s="18" t="inlineStr">
+      <c r="B8" s="17" t="inlineStr">
         <is>
           <t>24 body parts</t>
         </is>
       </c>
-      <c r="C8" s="20" t="inlineStr">
+      <c r="C8" s="19" t="inlineStr">
         <is>
           <t>576x768x3</t>
         </is>
       </c>
-      <c r="D8" s="20" t="n"/>
-      <c r="E8" s="20" t="n">
+      <c r="D8" s="19" t="n"/>
+      <c r="E8" s="19" t="n">
         <v>0.75</v>
       </c>
-      <c r="F8" s="20" t="n">
+      <c r="F8" s="19" t="n">
         <v>16</v>
       </c>
-      <c r="G8" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="H8" s="20" t="n">
+      <c r="G8" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" s="19" t="n">
         <v>17.7</v>
       </c>
-      <c r="I8" s="20" t="inlineStr">
+      <c r="I8" s="19" t="inlineStr">
         <is>
           <t>Yes*</t>
         </is>
       </c>
-      <c r="J8" s="20" t="inlineStr">
+      <c r="J8" s="19" t="inlineStr">
         <is>
           <t>1.8 MB</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="17.25" customHeight="1" s="15">
-      <c r="A9" s="18" t="inlineStr">
+    <row r="9" ht="17.25" customHeight="1" s="14">
+      <c r="A9" s="17" t="inlineStr">
         <is>
           <t>MobileNet v1 BodyPix</t>
         </is>
       </c>
-      <c r="B9" s="18" t="inlineStr">
+      <c r="B9" s="17" t="inlineStr">
         <is>
           <t>24 body parts</t>
         </is>
       </c>
-      <c r="C9" s="20" t="inlineStr">
+      <c r="C9" s="19" t="inlineStr">
         <is>
           <t>768x1024x3</t>
         </is>
       </c>
-      <c r="D9" s="20" t="n"/>
-      <c r="E9" s="20" t="n">
+      <c r="D9" s="19" t="n"/>
+      <c r="E9" s="19" t="n">
         <v>0.75</v>
       </c>
-      <c r="F9" s="20" t="n">
+      <c r="F9" s="19" t="n">
         <v>16</v>
       </c>
-      <c r="G9" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="H9" s="20" t="n">
+      <c r="G9" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="H9" s="19" t="n">
         <v>30.8</v>
       </c>
-      <c r="I9" s="20" t="inlineStr">
+      <c r="I9" s="19" t="inlineStr">
         <is>
           <t>Yes*</t>
         </is>
       </c>
-      <c r="J9" s="20" t="inlineStr">
+      <c r="J9" s="19" t="inlineStr">
         <is>
           <t>2.0 MB</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="17.25" customHeight="1" s="15">
-      <c r="A10" s="18" t="inlineStr">
+    <row r="10" ht="17.25" customHeight="1" s="14">
+      <c r="A10" s="17" t="inlineStr">
         <is>
           <t>MobileNet v1 BodyPix</t>
         </is>
       </c>
-      <c r="B10" s="18" t="inlineStr">
+      <c r="B10" s="17" t="inlineStr">
         <is>
           <t>24 body parts</t>
         </is>
       </c>
-      <c r="C10" s="20" t="inlineStr">
+      <c r="C10" s="19" t="inlineStr">
         <is>
           <t>720x1280x3</t>
         </is>
       </c>
-      <c r="D10" s="20" t="n"/>
-      <c r="E10" s="20" t="n">
+      <c r="D10" s="19" t="n"/>
+      <c r="E10" s="19" t="n">
         <v>0.75</v>
       </c>
-      <c r="F10" s="20" t="n">
+      <c r="F10" s="19" t="n">
         <v>16</v>
       </c>
-      <c r="G10" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="H10" s="20" t="n">
+      <c r="G10" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="H10" s="19" t="n">
         <v>38.8</v>
       </c>
-      <c r="I10" s="20" t="inlineStr">
+      <c r="I10" s="19" t="inlineStr">
         <is>
           <t>Yes*</t>
         </is>
       </c>
-      <c r="J10" s="20" t="inlineStr">
+      <c r="J10" s="19" t="inlineStr">
         <is>
           <t>2.3 MB</t>
         </is>
@@ -2493,134 +2396,134 @@
   <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="21.29" customWidth="1" style="14" min="1" max="1"/>
-    <col width="16.57" customWidth="1" style="14" min="2" max="3"/>
-    <col width="17.57" customWidth="1" style="14" min="6" max="6"/>
+    <col width="21.3" customWidth="1" style="13" min="1" max="1"/>
+    <col width="16.57" customWidth="1" style="13" min="2" max="3"/>
+    <col width="17.57" customWidth="1" style="13" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="70.5" customHeight="1" s="15">
-      <c r="A1" s="16" t="inlineStr">
+    <row r="1" ht="70.5" customHeight="1" s="14">
+      <c r="A1" s="15" t="inlineStr">
         <is>
           <t>Model name</t>
         </is>
       </c>
-      <c r="B1" s="16" t="inlineStr">
+      <c r="B1" s="15" t="inlineStr">
         <is>
           <t>Detections/Dataset</t>
         </is>
       </c>
-      <c r="C1" s="16" t="inlineStr">
+      <c r="C1" s="15" t="inlineStr">
         <is>
           <t>Input size</t>
         </is>
       </c>
-      <c r="D1" s="16" t="inlineStr">
+      <c r="D1" s="15" t="inlineStr">
         <is>
           <t>Micro 1</t>
         </is>
       </c>
-      <c r="E1" s="16" t="inlineStr">
+      <c r="E1" s="15" t="inlineStr">
         <is>
           <t>Model size</t>
         </is>
       </c>
-      <c r="F1" s="16" t="inlineStr">
+      <c r="F1" s="15" t="inlineStr">
         <is>
           <t>Downloads</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="70.5" customHeight="1" s="15">
-      <c r="A2" s="18" t="inlineStr">
+    <row r="2" ht="70.5" customHeight="1" s="14">
+      <c r="A2" s="17" t="inlineStr">
         <is>
           <t>YamNet without frontend</t>
         </is>
       </c>
-      <c r="B2" s="18" t="inlineStr">
+      <c r="B2" s="17" t="inlineStr">
         <is>
           <t>520+ sounds</t>
         </is>
       </c>
-      <c r="C2" s="20" t="inlineStr">
+      <c r="C2" s="19" t="inlineStr">
         <is>
           <t>96x64x1 (spectrogram)</t>
         </is>
       </c>
-      <c r="D2" s="20" t="inlineStr">
+      <c r="D2" s="19" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E2" s="20" t="inlineStr">
+      <c r="E2" s="19" t="inlineStr">
         <is>
           <t>4.1 MB</t>
         </is>
       </c>
-      <c r="F2" s="26" t="inlineStr">
+      <c r="F2" s="23" t="inlineStr">
         <is>
           <t>Edge TPU model,</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="70.5" customHeight="1" s="15">
-      <c r="A3" s="18" t="inlineStr">
+    <row r="3" ht="70.5" customHeight="1" s="14">
+      <c r="A3" s="17" t="inlineStr">
         <is>
           <t>Keyword Spotter v0.7</t>
         </is>
       </c>
-      <c r="B3" s="18" t="inlineStr">
+      <c r="B3" s="17" t="inlineStr">
         <is>
           <t>140+ speech phrases</t>
         </is>
       </c>
-      <c r="C3" s="20" t="inlineStr">
+      <c r="C3" s="19" t="inlineStr">
         <is>
           <t>198x32x1 (spectrogram)</t>
         </is>
       </c>
-      <c r="D3" s="20" t="inlineStr">
+      <c r="D3" s="19" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E3" s="20" t="inlineStr">
+      <c r="E3" s="19" t="inlineStr">
         <is>
           <t>578 KB</t>
         </is>
       </c>
-      <c r="F3" s="26" t="inlineStr">
+      <c r="F3" s="23" t="inlineStr">
         <is>
           <t>Edge TPU model,</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="70.5" customHeight="1" s="15">
-      <c r="A4" s="18" t="inlineStr">
+    <row r="4" ht="70.5" customHeight="1" s="14">
+      <c r="A4" s="17" t="inlineStr">
         <is>
           <t>Keyword Spotter v0.8</t>
         </is>
       </c>
-      <c r="B4" s="18" t="inlineStr">
+      <c r="B4" s="17" t="inlineStr">
         <is>
           <t>140+ speech phrases</t>
         </is>
       </c>
-      <c r="C4" s="20" t="inlineStr">
+      <c r="C4" s="19" t="inlineStr">
         <is>
           <t>198x32x1 (spectrogram)</t>
         </is>
       </c>
-      <c r="D4" s="20" t="inlineStr">
+      <c r="D4" s="19" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E4" s="20" t="inlineStr">
+      <c r="E4" s="19" t="inlineStr">
         <is>
           <t>578 KB</t>
         </is>
       </c>
-      <c r="F4" s="26" t="inlineStr">
+      <c r="F4" s="23" t="inlineStr">
         <is>
           <t>Edge TPU model,</t>
         </is>
@@ -2647,198 +2550,198 @@
   <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="23.15" customWidth="1" style="14" min="1" max="1"/>
-    <col width="16.43" customWidth="1" style="14" min="2" max="2"/>
-    <col width="17.14" customWidth="1" style="14" min="3" max="3"/>
-    <col width="14.43" customWidth="1" style="14" min="4" max="4"/>
-    <col width="13.43" customWidth="1" style="14" min="5" max="5"/>
-    <col width="18.43" customWidth="1" style="14" min="6" max="6"/>
-    <col width="13.29" customWidth="1" style="14" min="8" max="8"/>
+    <col width="23.15" customWidth="1" style="13" min="1" max="1"/>
+    <col width="16.43" customWidth="1" style="13" min="2" max="2"/>
+    <col width="17.14" customWidth="1" style="13" min="3" max="3"/>
+    <col width="14.43" customWidth="1" style="13" min="4" max="4"/>
+    <col width="13.43" customWidth="1" style="13" min="5" max="5"/>
+    <col width="18.43" customWidth="1" style="13" min="6" max="6"/>
+    <col width="13.3" customWidth="1" style="13" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="36" customHeight="1" s="15">
-      <c r="A1" s="16" t="inlineStr">
+    <row r="1" ht="36" customHeight="1" s="14">
+      <c r="A1" s="15" t="inlineStr">
         <is>
           <t>Model name</t>
         </is>
       </c>
-      <c r="B1" s="16" t="inlineStr">
+      <c r="B1" s="15" t="inlineStr">
         <is>
           <t>Detections/Dataset</t>
         </is>
       </c>
-      <c r="C1" s="16" t="inlineStr">
+      <c r="C1" s="15" t="inlineStr">
         <is>
           <t>Input size</t>
         </is>
       </c>
-      <c r="D1" s="16" t="inlineStr">
+      <c r="D1" s="15" t="inlineStr">
         <is>
           <t>Output stride</t>
         </is>
       </c>
-      <c r="E1" s="16" t="inlineStr">
+      <c r="E1" s="15" t="inlineStr">
         <is>
           <t>TF ver.</t>
         </is>
       </c>
-      <c r="F1" s="17" t="inlineStr">
+      <c r="F1" s="16" t="inlineStr">
         <is>
           <t>Latency (ms) 1</t>
         </is>
       </c>
-      <c r="G1" s="16" t="inlineStr">
+      <c r="G1" s="15" t="inlineStr">
         <is>
           <t>Micro 2</t>
         </is>
       </c>
-      <c r="H1" s="16" t="inlineStr">
+      <c r="H1" s="15" t="inlineStr">
         <is>
           <t>Model size</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="36" customHeight="1" s="15">
-      <c r="A2" s="24" t="inlineStr">
+    <row r="2" ht="36" customHeight="1" s="14">
+      <c r="A2" s="21" t="inlineStr">
         <is>
           <t>PoseNet MobileNet V1</t>
         </is>
       </c>
-      <c r="B2" s="24" t="inlineStr">
+      <c r="B2" s="21" t="inlineStr">
         <is>
           <t>17 body points</t>
         </is>
       </c>
-      <c r="C2" s="25" t="inlineStr">
+      <c r="C2" s="22" t="inlineStr">
         <is>
           <t>324x324x3</t>
         </is>
       </c>
-      <c r="D2" s="25" t="n">
+      <c r="D2" s="22" t="n">
         <v>16</v>
       </c>
-      <c r="E2" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="F2" s="25" t="inlineStr">
+      <c r="E2" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" s="22" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="G2" s="25" t="inlineStr">
+      <c r="G2" s="22" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="H2" s="25" t="inlineStr">
+      <c r="H2" s="22" t="inlineStr">
         <is>
           <t>1.6 MB</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="36" customHeight="1" s="15">
-      <c r="A3" s="18" t="inlineStr">
+    <row r="3" ht="36" customHeight="1" s="14">
+      <c r="A3" s="17" t="inlineStr">
         <is>
           <t>PoseNet MobileNet V1</t>
         </is>
       </c>
-      <c r="B3" s="18" t="inlineStr">
+      <c r="B3" s="17" t="inlineStr">
         <is>
           <t>17 body points</t>
         </is>
       </c>
-      <c r="C3" s="20" t="inlineStr">
+      <c r="C3" s="19" t="inlineStr">
         <is>
           <t>353x481x3</t>
         </is>
       </c>
-      <c r="D3" s="20" t="n">
+      <c r="D3" s="19" t="n">
         <v>16</v>
       </c>
-      <c r="E3" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="F3" s="20" t="n">
+      <c r="E3" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" s="19" t="n">
         <v>5.8</v>
       </c>
-      <c r="G3" s="20" t="inlineStr">
+      <c r="G3" s="19" t="inlineStr">
         <is>
           <t>Yes*</t>
         </is>
       </c>
-      <c r="H3" s="20" t="inlineStr">
+      <c r="H3" s="19" t="inlineStr">
         <is>
           <t>1.5 MB</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="36" customHeight="1" s="15">
-      <c r="A4" s="18" t="inlineStr">
+    <row r="4" ht="36" customHeight="1" s="14">
+      <c r="A4" s="17" t="inlineStr">
         <is>
           <t>PoseNet MobileNet V1</t>
         </is>
       </c>
-      <c r="B4" s="18" t="inlineStr">
+      <c r="B4" s="17" t="inlineStr">
         <is>
           <t>17 body points</t>
         </is>
       </c>
-      <c r="C4" s="20" t="inlineStr">
+      <c r="C4" s="19" t="inlineStr">
         <is>
           <t>481x641x3</t>
         </is>
       </c>
-      <c r="D4" s="20" t="n">
+      <c r="D4" s="19" t="n">
         <v>16</v>
       </c>
-      <c r="E4" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="F4" s="20" t="n">
+      <c r="E4" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" s="19" t="n">
         <v>10.3</v>
       </c>
-      <c r="G4" s="20" t="inlineStr">
+      <c r="G4" s="19" t="inlineStr">
         <is>
           <t>Yes*</t>
         </is>
       </c>
-      <c r="H4" s="20" t="inlineStr">
+      <c r="H4" s="19" t="inlineStr">
         <is>
           <t>1.7 MB</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="36" customHeight="1" s="15">
-      <c r="A5" s="18" t="inlineStr">
+    <row r="5" ht="36" customHeight="1" s="14">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>PoseNet MobileNet V1</t>
         </is>
       </c>
-      <c r="B5" s="18" t="inlineStr">
+      <c r="B5" s="17" t="inlineStr">
         <is>
           <t>17 body points</t>
         </is>
       </c>
-      <c r="C5" s="20" t="inlineStr">
+      <c r="C5" s="19" t="inlineStr">
         <is>
           <t>721x1281x3</t>
         </is>
       </c>
-      <c r="D5" s="20" t="n">
+      <c r="D5" s="19" t="n">
         <v>16</v>
       </c>
-      <c r="E5" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="F5" s="20" t="n">
+      <c r="E5" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" s="19" t="n">
         <v>32.4</v>
       </c>
-      <c r="G5" s="20" t="inlineStr">
+      <c r="G5" s="19" t="inlineStr">
         <is>
           <t>Yes*</t>
         </is>
       </c>
-      <c r="H5" s="20" t="inlineStr">
+      <c r="H5" s="19" t="inlineStr">
         <is>
           <t>2.5 MB</t>
         </is>
@@ -2861,27 +2764,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="23" t="inlineStr">
+      <c r="A1" s="20" t="inlineStr">
         <is>
           <t>Model Name</t>
         </is>
       </c>
-      <c r="B1" s="23" t="inlineStr">
+      <c r="B1" s="20" t="inlineStr">
         <is>
           <t>Latency (ms)</t>
         </is>
       </c>
-      <c r="C1" s="23" t="inlineStr">
+      <c r="C1" s="20" t="inlineStr">
         <is>
           <t>Measured Inference Time (ms)</t>
         </is>
       </c>
-      <c r="D1" s="23" t="inlineStr">
+      <c r="D1" s="20" t="inlineStr">
         <is>
           <t>mAP</t>
         </is>
       </c>
-      <c r="E1" s="23" t="inlineStr">
+      <c r="E1" s="20" t="inlineStr">
         <is>
           <t>Parameter Count (M)</t>
         </is>
@@ -2903,7 +2806,7 @@
         <v>22.4</v>
       </c>
       <c r="E2" t="n">
-        <v>6.814845</v>
+        <v>6.055325</v>
       </c>
     </row>
     <row r="3">
@@ -2922,7 +2825,7 @@
         <v>21.5</v>
       </c>
       <c r="E3" t="n">
-        <v>6.055325</v>
+        <v>4.129913</v>
       </c>
     </row>
     <row r="4">
@@ -2941,7 +2844,7 @@
         <v>25.6</v>
       </c>
       <c r="E4" t="n">
-        <v>6.055325</v>
+        <v>6.814845</v>
       </c>
     </row>
     <row r="5">
@@ -2960,7 +2863,7 @@
         <v>32.9</v>
       </c>
       <c r="E5" t="n">
-        <v>4.129913</v>
+        <v>6.055325</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
added way to plot specific models by name from a run directory containing many models
</commit_message>
<xml_diff>
--- a/scripts/Model_Stats.xlsx
+++ b/scripts/Model_Stats.xlsx
@@ -1268,289 +1268,289 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="13" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>MobileNet V1 (0.25)</t>
         </is>
       </c>
-      <c r="B2" s="13" t="n">
+      <c r="B2" t="n">
         <v>0.9</v>
       </c>
-      <c r="C2" s="13" t="n">
+      <c r="C2" t="n">
         <v>40.8</v>
       </c>
-      <c r="D2" s="13" t="n">
+      <c r="D2" t="n">
         <v>95.09999999999999</v>
       </c>
-      <c r="E2" s="13" t="n">
-        <v>4.273343636746742</v>
-      </c>
-      <c r="F2" s="13" t="n">
+      <c r="E2" t="n">
+        <v>8.615658759558197</v>
+      </c>
+      <c r="F2" t="n">
         <v>0.467595</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>MobileNet V1 (0.50)</t>
         </is>
       </c>
-      <c r="B3" s="13" t="n">
+      <c r="B3" t="n">
         <v>1.4</v>
       </c>
-      <c r="C3" s="13" t="n">
+      <c r="C3" t="n">
         <v>63.7</v>
       </c>
-      <c r="D3" s="13" t="n">
+      <c r="D3" t="n">
         <v>94.5</v>
       </c>
-      <c r="E3" s="13" t="n">
-        <v>5.741725413576729</v>
-      </c>
-      <c r="F3" s="13" t="n">
+      <c r="E3" t="n">
+        <v>11.45077828213879</v>
+      </c>
+      <c r="F3" t="n">
         <v>1.326635</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="inlineStr">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>MobileNet V1 (.75)</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="C4" t="n">
+        <v>67.2</v>
+      </c>
+      <c r="D4" t="n">
+        <v>94.7</v>
+      </c>
+      <c r="E4" t="n">
+        <v>13.00876647286822</v>
+      </c>
+      <c r="F4" t="n">
+        <v>2.578123</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
         <is>
           <t>MobileNet V1 (1.0)</t>
         </is>
       </c>
-      <c r="B4" s="13" t="n">
+      <c r="B5" t="n">
         <v>2.8</v>
       </c>
-      <c r="C4" s="13" t="n">
+      <c r="C5" t="n">
         <v>69.5</v>
       </c>
-      <c r="D4" s="13" t="n">
-        <v>94.7</v>
-      </c>
-      <c r="E4" s="13" t="n">
-        <v>6.408314722753338</v>
-      </c>
-      <c r="F4" s="13" t="n">
+      <c r="D5" t="n">
+        <v>92</v>
+      </c>
+      <c r="E5" t="n">
+        <v>15.09704858858859</v>
+      </c>
+      <c r="F5" t="n">
         <v>4.899478</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="13" t="inlineStr">
-        <is>
-          <t>MobileNet V1 (.75)</t>
-        </is>
-      </c>
-      <c r="B5" s="13" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="C5" s="13" t="n">
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>MobileNet V2</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="C6" t="n">
+        <v>73.2</v>
+      </c>
+      <c r="D6" t="n">
+        <v>93.2</v>
+      </c>
+      <c r="E6" t="n">
+        <v>17.11049792869269</v>
+      </c>
+      <c r="F6" t="n">
+        <v>3.489099</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>MobileNet V1 (TF_ver_2.0)</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="C7" t="n">
+        <v>69.5</v>
+      </c>
+      <c r="D7" t="n">
         <v>67.2</v>
       </c>
-      <c r="D5" s="13" t="n">
-        <v>92</v>
-      </c>
-      <c r="E5" s="13" t="n">
-        <v>6.413245242038233</v>
-      </c>
-      <c r="F5" s="13" t="n">
-        <v>2.578123</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="13" t="inlineStr">
-        <is>
-          <t>MobileNet V2</t>
-        </is>
-      </c>
-      <c r="B6" s="13" t="n">
-        <v>2.9</v>
-      </c>
-      <c r="C6" s="13" t="n">
+      <c r="E7" t="n">
+        <v>18.45211108058609</v>
+      </c>
+      <c r="F7" t="n">
+        <v>4.222061</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>MobileNet V2 (TF_ver_2.0)</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>3</v>
+      </c>
+      <c r="C8" t="n">
         <v>73.2</v>
       </c>
-      <c r="D6" s="13" t="n">
-        <v>93.2</v>
-      </c>
-      <c r="E6" s="13" t="n">
-        <v>7.892005935786992</v>
-      </c>
-      <c r="F6" s="13" t="n">
-        <v>3.489099</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="13" t="inlineStr">
-        <is>
-          <t>MobileNet V2 (TF_ver_2.0)</t>
-        </is>
-      </c>
-      <c r="B7" s="13" t="n">
+      <c r="D8" t="n">
+        <v>83.40000000000001</v>
+      </c>
+      <c r="E8" t="n">
+        <v>18.60979228200372</v>
+      </c>
+      <c r="F8" t="n">
+        <v>3.489101</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>MobileNet V3</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
         <v>3</v>
       </c>
-      <c r="C7" s="13" t="n">
-        <v>73.2</v>
-      </c>
-      <c r="D7" s="13" t="n">
-        <v>67.2</v>
-      </c>
-      <c r="E7" s="13" t="n">
-        <v>8.365876630525435</v>
-      </c>
-      <c r="F7" s="13" t="n">
-        <v>3.489101</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="13" t="inlineStr">
-        <is>
-          <t>MobileNet V1 (TF_ver_2.0)</t>
-        </is>
-      </c>
-      <c r="B8" s="13" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="C8" s="13" t="n">
-        <v>69.5</v>
-      </c>
-      <c r="D8" s="13" t="n">
-        <v>83.40000000000001</v>
-      </c>
-      <c r="E8" s="13" t="n">
-        <v>8.588968593350385</v>
-      </c>
-      <c r="F8" s="13" t="n">
-        <v>4.222061</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="13" t="inlineStr">
-        <is>
-          <t>MobileNet V3</t>
-        </is>
-      </c>
-      <c r="B9" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="C9" s="13" t="n">
+      <c r="C9" t="n">
         <v>77.5</v>
       </c>
-      <c r="D9" s="13" t="n">
+      <c r="D9" t="n">
         <v>88.09999999999999</v>
       </c>
-      <c r="E9" s="13" t="n">
-        <v>8.700641511226253</v>
-      </c>
-      <c r="F9" s="13" t="n">
+      <c r="E9" t="n">
+        <v>19.01006683018869</v>
+      </c>
+      <c r="F9" t="n">
         <v>4.073277</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="13" t="inlineStr">
+      <c r="A10" t="inlineStr">
         <is>
           <t>EfficientNet-EdgeTpu (S)</t>
         </is>
       </c>
-      <c r="B10" s="13" t="n">
+      <c r="B10" t="n">
         <v>5</v>
       </c>
-      <c r="C10" s="13" t="n">
+      <c r="C10" t="n">
         <v>78.90000000000001</v>
       </c>
-      <c r="D10" s="13" t="n">
+      <c r="D10" t="n">
         <v>90.59999999999999</v>
       </c>
-      <c r="E10" s="13" t="n">
-        <v>9.05769085895118</v>
-      </c>
-      <c r="F10" s="13" t="n">
+      <c r="E10" t="n">
+        <v>20.11606214859438</v>
+      </c>
+      <c r="F10" t="n">
         <v>5.413955</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="13" t="inlineStr">
+      <c r="A11" t="inlineStr">
         <is>
           <t>Inception V1</t>
         </is>
       </c>
-      <c r="B11" s="13" t="n">
+      <c r="B11" t="n">
         <v>3.4</v>
       </c>
-      <c r="C11" s="13" t="n">
+      <c r="C11" t="n">
         <v>71.90000000000001</v>
       </c>
-      <c r="D11" s="13" t="n">
+      <c r="D11" t="n">
         <v>89.8</v>
       </c>
-      <c r="E11" s="13" t="n">
-        <v>15.37397241960187</v>
-      </c>
-      <c r="F11" s="13" t="n">
+      <c r="E11" t="n">
+        <v>33.13267303630368</v>
+      </c>
+      <c r="F11" t="n">
         <v>6.618651</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="13" t="inlineStr">
+      <c r="A12" t="inlineStr">
         <is>
           <t>EfficientNet-EdgeTpu (M)</t>
         </is>
       </c>
-      <c r="B12" s="13" t="n">
+      <c r="B12" t="n">
         <v>7.3</v>
       </c>
-      <c r="C12" s="13" t="n">
+      <c r="C12" t="n">
         <v>80.09999999999999</v>
       </c>
-      <c r="D12" s="13" t="n">
+      <c r="D12" t="n">
         <v>90</v>
       </c>
-      <c r="E12" s="13" t="n">
-        <v>26.50050885333329</v>
-      </c>
-      <c r="F12" s="13" t="n">
+      <c r="E12" t="n">
+        <v>54.90435629834248</v>
+      </c>
+      <c r="F12" t="n">
         <v>6.866875</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="13" t="inlineStr">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Inception V3</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="C13" t="n">
+        <v>75.40000000000001</v>
+      </c>
+      <c r="D13" t="n">
+        <v>91.8</v>
+      </c>
+      <c r="E13" t="n">
+        <v>213.8618108695652</v>
+      </c>
+      <c r="F13" t="n">
+        <v>11.179387</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>EfficientNet-EdgeTpu (L)</t>
         </is>
       </c>
-      <c r="B13" s="13" t="n">
+      <c r="B14" t="n">
         <v>21.3</v>
       </c>
-      <c r="C13" s="13" t="n">
+      <c r="C14" t="n">
         <v>81.2</v>
       </c>
-      <c r="D13" s="13" t="n">
-        <v>91.8</v>
-      </c>
-      <c r="E13" s="13" t="n">
-        <v>102.4790272164949</v>
-      </c>
-      <c r="F13" s="13" t="n">
+      <c r="D14" t="n">
+        <v>93.59999999999999</v>
+      </c>
+      <c r="E14" t="n">
+        <v>225.9196586363637</v>
+      </c>
+      <c r="F14" t="n">
         <v>10.545147</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="13" t="inlineStr">
-        <is>
-          <t>Inception V3</t>
-        </is>
-      </c>
-      <c r="B14" s="13" t="n">
-        <v>13.4</v>
-      </c>
-      <c r="C14" s="13" t="n">
-        <v>75.40000000000001</v>
-      </c>
-      <c r="D14" s="13" t="n">
-        <v>93.59999999999999</v>
-      </c>
-      <c r="E14" s="13" t="n">
-        <v>118.5258274698795</v>
-      </c>
-      <c r="F14" s="13" t="n">
-        <v>11.179387</v>
       </c>
     </row>
   </sheetData>
@@ -2791,95 +2791,95 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="13" t="inlineStr">
         <is>
           <t>SSD MobileNet V2 (TF2)</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" s="13" t="n">
         <v>7.6</v>
       </c>
-      <c r="C2" t="n">
+      <c r="C2" s="13" t="n">
         <v>17.35170945392494</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" s="13" t="n">
         <v>22.4</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2" s="13" t="n">
         <v>6.055325</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="13" t="inlineStr">
         <is>
           <t>SSD MobileNet V1</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" s="13" t="n">
         <v>6.5</v>
       </c>
-      <c r="C3" t="n">
+      <c r="C3" s="13" t="n">
         <v>36.54455787545788</v>
       </c>
-      <c r="D3" t="n">
+      <c r="D3" s="13" t="n">
         <v>21.5</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E3" s="13" t="n">
         <v>4.129913</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="13" t="inlineStr">
         <is>
           <t>SSD MobileNet V2(TF1)</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" s="13" t="n">
         <v>7.3</v>
       </c>
-      <c r="C4" t="n">
+      <c r="C4" s="13" t="n">
         <v>39.4892774015748</v>
       </c>
-      <c r="D4" t="n">
+      <c r="D4" s="13" t="n">
         <v>25.6</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E4" s="13" t="n">
         <v>6.814845</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="13" t="inlineStr">
         <is>
           <t>SSDLite MobileDet</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" s="13" t="n">
         <v>9.1</v>
       </c>
-      <c r="C5" t="n">
+      <c r="C5" s="13" t="n">
         <v>41.2180785185186</v>
       </c>
-      <c r="D5" t="n">
+      <c r="D5" s="13" t="n">
         <v>32.9</v>
       </c>
-      <c r="E5" t="n">
+      <c r="E5" s="13" t="n">
         <v>6.055325</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="13" t="inlineStr">
         <is>
           <t>SSD MobileNet V2</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="B6" s="13" t="n">
         <v>5.2</v>
       </c>
-      <c r="C6" t="n">
+      <c r="C6" s="13" t="n">
         <v>70.80963588652483</v>
       </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="n">
+      <c r="D6" s="13" t="inlineStr"/>
+      <c r="E6" s="13" t="n">
         <v>5.383744</v>
       </c>
     </row>

</xml_diff>